<commit_message>
data: nifty500 scan 2026-06-26 09:31 IST
</commit_message>
<xml_diff>
--- a/data/nifty500_latest.xlsx
+++ b/data/nifty500_latest.xlsx
@@ -794,7 +794,7 @@
         <v>42.79</v>
       </c>
       <c r="AQ2" t="n">
-        <v>50.23</v>
+        <v>50.51</v>
       </c>
       <c r="AR2" t="n">
         <v>1110.95</v>
@@ -812,157 +812,51 @@
           <t>3MINDIA.NS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Diversified</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>33225</v>
-      </c>
-      <c r="F3" t="n">
-        <v>33225</v>
-      </c>
-      <c r="G3" t="n">
-        <v>32810</v>
-      </c>
-      <c r="H3" t="n">
-        <v>32560</v>
-      </c>
-      <c r="I3" t="n">
-        <v>32610</v>
-      </c>
-      <c r="J3" t="n">
-        <v>32445</v>
-      </c>
-      <c r="K3" t="n">
-        <v>32290</v>
-      </c>
-      <c r="L3" t="n">
-        <v>31995</v>
-      </c>
-      <c r="M3" t="n">
-        <v>31540</v>
-      </c>
-      <c r="N3" t="n">
-        <v>31785</v>
-      </c>
-      <c r="O3" t="n">
-        <v>31580</v>
-      </c>
-      <c r="P3" t="n">
-        <v>31165</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>31550</v>
-      </c>
-      <c r="R3" t="n">
-        <v>31665</v>
-      </c>
-      <c r="S3" t="n">
-        <v>32300</v>
-      </c>
-      <c r="T3" t="n">
-        <v>33060</v>
-      </c>
-      <c r="U3" t="n">
-        <v>33250</v>
-      </c>
-      <c r="V3" t="n">
-        <v>33125</v>
-      </c>
-      <c r="W3" t="n">
-        <v>33325</v>
-      </c>
-      <c r="X3" t="n">
-        <v>33615</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>33535</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>33380</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>32507.38</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>2.68</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>33615</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>31165</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>7.11</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>7.86</v>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>Between</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>Doji</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>Shooting Star</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="n">
-        <v>-0.46</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>62.21</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>53.35</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>33070.11</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>32265.96</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>2.49</v>
-      </c>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1110,7 +1004,7 @@
         <v>66.73</v>
       </c>
       <c r="AQ4" t="n">
-        <v>63.59</v>
+        <v>63.43</v>
       </c>
       <c r="AR4" t="n">
         <v>497.94</v>
@@ -1268,7 +1162,7 @@
         <v>47.47</v>
       </c>
       <c r="AQ5" t="n">
-        <v>55.38</v>
+        <v>55.43</v>
       </c>
       <c r="AR5" t="n">
         <v>472.45</v>
@@ -1426,7 +1320,7 @@
         <v>70.94</v>
       </c>
       <c r="AQ6" t="n">
-        <v>60.77</v>
+        <v>60.99</v>
       </c>
       <c r="AR6" t="n">
         <v>1447.81</v>
@@ -1584,7 +1478,7 @@
         <v>48.46</v>
       </c>
       <c r="AQ7" t="n">
-        <v>57.5</v>
+        <v>57.2</v>
       </c>
       <c r="AR7" t="n">
         <v>7068.83</v>
@@ -1742,7 +1636,7 @@
         <v>35.4</v>
       </c>
       <c r="AQ8" t="n">
-        <v>38.91</v>
+        <v>39.39</v>
       </c>
       <c r="AR8" t="n">
         <v>25883.27</v>
@@ -1900,7 +1794,7 @@
         <v>65.02</v>
       </c>
       <c r="AQ9" t="n">
-        <v>71.5</v>
+        <v>71.81</v>
       </c>
       <c r="AR9" t="n">
         <v>380.2</v>
@@ -2058,7 +1952,7 @@
         <v>63.78</v>
       </c>
       <c r="AQ10" t="n">
-        <v>61.82</v>
+        <v>62.16</v>
       </c>
       <c r="AR10" t="n">
         <v>617.74</v>
@@ -2216,7 +2110,7 @@
         <v>44.89</v>
       </c>
       <c r="AQ11" t="n">
-        <v>41.28</v>
+        <v>41.03</v>
       </c>
       <c r="AR11" t="n">
         <v>60.65</v>
@@ -2374,7 +2268,7 @@
         <v>44.86</v>
       </c>
       <c r="AQ12" t="n">
-        <v>40.21</v>
+        <v>40.06</v>
       </c>
       <c r="AR12" t="n">
         <v>98.61</v>
@@ -2532,7 +2426,7 @@
         <v>62.44</v>
       </c>
       <c r="AQ13" t="n">
-        <v>50.15</v>
+        <v>49.39</v>
       </c>
       <c r="AR13" t="n">
         <v>1298.59</v>
@@ -2690,7 +2584,7 @@
         <v>55.29</v>
       </c>
       <c r="AQ14" t="n">
-        <v>67.19</v>
+        <v>68.16</v>
       </c>
       <c r="AR14" t="n">
         <v>1153.19</v>
@@ -2848,7 +2742,7 @@
         <v>46.93</v>
       </c>
       <c r="AQ15" t="n">
-        <v>33.46</v>
+        <v>33.21</v>
       </c>
       <c r="AR15" t="n">
         <v>1341.83</v>
@@ -3006,7 +2900,7 @@
         <v>66.58</v>
       </c>
       <c r="AQ16" t="n">
-        <v>62.38</v>
+        <v>62.03</v>
       </c>
       <c r="AR16" t="n">
         <v>975.4299999999999</v>
@@ -3164,7 +3058,7 @@
         <v>67.3</v>
       </c>
       <c r="AQ17" t="n">
-        <v>71.03</v>
+        <v>71.16</v>
       </c>
       <c r="AR17" t="n">
         <v>347.42</v>
@@ -3322,7 +3216,7 @@
         <v>65.59</v>
       </c>
       <c r="AQ18" t="n">
-        <v>74.76000000000001</v>
+        <v>74.67</v>
       </c>
       <c r="AR18" t="n">
         <v>3217.33</v>
@@ -3480,7 +3374,7 @@
         <v>53.58</v>
       </c>
       <c r="AQ19" t="n">
-        <v>69.11</v>
+        <v>68.94</v>
       </c>
       <c r="AR19" t="n">
         <v>1506.84</v>
@@ -3638,7 +3532,7 @@
         <v>60.84</v>
       </c>
       <c r="AQ20" t="n">
-        <v>74.77</v>
+        <v>74.84</v>
       </c>
       <c r="AR20" t="n">
         <v>3008.53</v>
@@ -3796,7 +3690,7 @@
         <v>59.85</v>
       </c>
       <c r="AQ21" t="n">
-        <v>77.42</v>
+        <v>77.41</v>
       </c>
       <c r="AR21" t="n">
         <v>1509.99</v>
@@ -3954,7 +3848,7 @@
         <v>48.98</v>
       </c>
       <c r="AQ22" t="n">
-        <v>69.15000000000001</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="AR22" t="n">
         <v>1810.5</v>
@@ -4112,7 +4006,7 @@
         <v>52.49</v>
       </c>
       <c r="AQ23" t="n">
-        <v>68.65000000000001</v>
+        <v>68.52</v>
       </c>
       <c r="AR23" t="n">
         <v>228.84</v>
@@ -4270,7 +4164,7 @@
         <v>90.31</v>
       </c>
       <c r="AQ24" t="n">
-        <v>85.53</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="AR24" t="n">
         <v>1029.61</v>
@@ -4428,7 +4322,7 @@
         <v>61.89</v>
       </c>
       <c r="AQ25" t="n">
-        <v>58.5</v>
+        <v>58.85</v>
       </c>
       <c r="AR25" t="n">
         <v>231.15</v>
@@ -4586,7 +4480,7 @@
         <v>49.83</v>
       </c>
       <c r="AQ26" t="n">
-        <v>46.72</v>
+        <v>46.67</v>
       </c>
       <c r="AR26" t="n">
         <v>317.72</v>
@@ -4744,7 +4638,7 @@
         <v>44.32</v>
       </c>
       <c r="AQ27" t="n">
-        <v>44.9</v>
+        <v>44.6</v>
       </c>
       <c r="AR27" t="n">
         <v>1465.67</v>
@@ -4902,7 +4796,7 @@
         <v>72.53</v>
       </c>
       <c r="AQ28" t="n">
-        <v>71.23</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="AR28" t="n">
         <v>4713.54</v>
@@ -5060,7 +4954,7 @@
         <v>51.37</v>
       </c>
       <c r="AQ29" t="n">
-        <v>52.97</v>
+        <v>52.5</v>
       </c>
       <c r="AR29" t="n">
         <v>529.97</v>
@@ -5218,7 +5112,7 @@
         <v>60</v>
       </c>
       <c r="AQ30" t="n">
-        <v>63.87</v>
+        <v>64.27</v>
       </c>
       <c r="AR30" t="n">
         <v>3146.85</v>
@@ -5534,7 +5428,7 @@
         <v>47.16</v>
       </c>
       <c r="AQ32" t="n">
-        <v>51.4</v>
+        <v>51.2</v>
       </c>
       <c r="AR32" t="n">
         <v>7770.39</v>
@@ -5692,7 +5586,7 @@
         <v>48.43</v>
       </c>
       <c r="AQ33" t="n">
-        <v>37.23</v>
+        <v>37.32</v>
       </c>
       <c r="AR33" t="n">
         <v>423.75</v>
@@ -5850,7 +5744,7 @@
         <v>77.02</v>
       </c>
       <c r="AQ34" t="n">
-        <v>74.93000000000001</v>
+        <v>75.20999999999999</v>
       </c>
       <c r="AR34" t="n">
         <v>1867.27</v>
@@ -6008,7 +5902,7 @@
         <v>47.5</v>
       </c>
       <c r="AQ35" t="n">
-        <v>50.33</v>
+        <v>50.13</v>
       </c>
       <c r="AR35" t="n">
         <v>527.9299999999999</v>
@@ -6166,7 +6060,7 @@
         <v>46.38</v>
       </c>
       <c r="AQ36" t="n">
-        <v>61.93</v>
+        <v>62.02</v>
       </c>
       <c r="AR36" t="n">
         <v>343.19</v>
@@ -6324,7 +6218,7 @@
         <v>46.08</v>
       </c>
       <c r="AQ37" t="n">
-        <v>57.42</v>
+        <v>57.34</v>
       </c>
       <c r="AR37" t="n">
         <v>770.78</v>
@@ -6482,7 +6376,7 @@
         <v>42.83</v>
       </c>
       <c r="AQ38" t="n">
-        <v>47.76</v>
+        <v>46.93</v>
       </c>
       <c r="AR38" t="n">
         <v>1279.37</v>
@@ -6640,7 +6534,7 @@
         <v>64.14</v>
       </c>
       <c r="AQ39" t="n">
-        <v>79.93000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="AR39" t="n">
         <v>15970.25</v>
@@ -6798,7 +6692,7 @@
         <v>38.17</v>
       </c>
       <c r="AQ40" t="n">
-        <v>39.16</v>
+        <v>39.58</v>
       </c>
       <c r="AR40" t="n">
         <v>1829.83</v>
@@ -6956,7 +6850,7 @@
         <v>69.38</v>
       </c>
       <c r="AQ41" t="n">
-        <v>71.36</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="AR41" t="n">
         <v>8495.629999999999</v>
@@ -7114,7 +7008,7 @@
         <v>66.22</v>
       </c>
       <c r="AQ42" t="n">
-        <v>51.54</v>
+        <v>51.52</v>
       </c>
       <c r="AR42" t="n">
         <v>420.79</v>
@@ -7272,7 +7166,7 @@
         <v>50.7</v>
       </c>
       <c r="AQ43" t="n">
-        <v>54.72</v>
+        <v>54.66</v>
       </c>
       <c r="AR43" t="n">
         <v>266.29</v>
@@ -7430,7 +7324,7 @@
         <v>46.07</v>
       </c>
       <c r="AQ44" t="n">
-        <v>48.66</v>
+        <v>48.69</v>
       </c>
       <c r="AR44" t="n">
         <v>843.4400000000001</v>
@@ -7588,7 +7482,7 @@
         <v>59.14</v>
       </c>
       <c r="AQ45" t="n">
-        <v>54.25</v>
+        <v>54.93</v>
       </c>
       <c r="AR45" t="n">
         <v>873.61</v>
@@ -7746,7 +7640,7 @@
         <v>60.18</v>
       </c>
       <c r="AQ46" t="n">
-        <v>49.19</v>
+        <v>49.46</v>
       </c>
       <c r="AR46" t="n">
         <v>155.52</v>
@@ -7904,7 +7798,7 @@
         <v>46.39</v>
       </c>
       <c r="AQ47" t="n">
-        <v>59.22</v>
+        <v>58.71</v>
       </c>
       <c r="AR47" t="n">
         <v>2675.04</v>
@@ -8062,7 +7956,7 @@
         <v>48.91</v>
       </c>
       <c r="AQ48" t="n">
-        <v>61.57</v>
+        <v>61.56</v>
       </c>
       <c r="AR48" t="n">
         <v>778.26</v>
@@ -8220,7 +8114,7 @@
         <v>38.78</v>
       </c>
       <c r="AQ49" t="n">
-        <v>42.55</v>
+        <v>42.88</v>
       </c>
       <c r="AR49" t="n">
         <v>1529.89</v>
@@ -8378,7 +8272,7 @@
         <v>51.4</v>
       </c>
       <c r="AQ50" t="n">
-        <v>65.01000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="AR50" t="n">
         <v>721.96</v>
@@ -8536,7 +8430,7 @@
         <v>53.65</v>
       </c>
       <c r="AQ51" t="n">
-        <v>66.09</v>
+        <v>66.06999999999999</v>
       </c>
       <c r="AR51" t="n">
         <v>992.58</v>
@@ -8694,7 +8588,7 @@
         <v>52.99</v>
       </c>
       <c r="AQ52" t="n">
-        <v>54.24</v>
+        <v>55.49</v>
       </c>
       <c r="AR52" t="n">
         <v>6577.98</v>
@@ -8852,7 +8746,7 @@
         <v>56.02</v>
       </c>
       <c r="AQ53" t="n">
-        <v>58.41</v>
+        <v>59.07</v>
       </c>
       <c r="AR53" t="n">
         <v>1030.24</v>
@@ -9010,7 +8904,7 @@
         <v>70.04000000000001</v>
       </c>
       <c r="AQ54" t="n">
-        <v>75.20999999999999</v>
+        <v>75.17</v>
       </c>
       <c r="AR54" t="n">
         <v>1498.53</v>
@@ -9168,7 +9062,7 @@
         <v>37.13</v>
       </c>
       <c r="AQ55" t="n">
-        <v>34.87</v>
+        <v>34.72</v>
       </c>
       <c r="AR55" t="n">
         <v>185.98</v>
@@ -9484,7 +9378,7 @@
         <v>38.36</v>
       </c>
       <c r="AQ57" t="n">
-        <v>51.78</v>
+        <v>51.93</v>
       </c>
       <c r="AR57" t="n">
         <v>9987.299999999999</v>
@@ -9642,7 +9536,7 @@
         <v>53.14</v>
       </c>
       <c r="AQ58" t="n">
-        <v>45.53</v>
+        <v>45.73</v>
       </c>
       <c r="AR58" t="n">
         <v>1761.14</v>
@@ -9800,7 +9694,7 @@
         <v>58.7</v>
       </c>
       <c r="AQ59" t="n">
-        <v>49.95</v>
+        <v>50.52</v>
       </c>
       <c r="AR59" t="n">
         <v>87</v>
@@ -9958,7 +9852,7 @@
         <v>55.92</v>
       </c>
       <c r="AQ60" t="n">
-        <v>52.87</v>
+        <v>53.39</v>
       </c>
       <c r="AR60" t="n">
         <v>10555.23</v>
@@ -10116,7 +10010,7 @@
         <v>66.72</v>
       </c>
       <c r="AQ61" t="n">
-        <v>58.44</v>
+        <v>58.58</v>
       </c>
       <c r="AR61" t="n">
         <v>960.42</v>
@@ -10274,7 +10168,7 @@
         <v>56.72</v>
       </c>
       <c r="AQ62" t="n">
-        <v>50.3</v>
+        <v>50.4</v>
       </c>
       <c r="AR62" t="n">
         <v>2213.4</v>
@@ -10432,7 +10326,7 @@
         <v>47.41</v>
       </c>
       <c r="AQ63" t="n">
-        <v>64.45999999999999</v>
+        <v>63.74</v>
       </c>
       <c r="AR63" t="n">
         <v>538.6799999999999</v>
@@ -10590,7 +10484,7 @@
         <v>45.17</v>
       </c>
       <c r="AQ64" t="n">
-        <v>62.32</v>
+        <v>62.65</v>
       </c>
       <c r="AR64" t="n">
         <v>207.71</v>
@@ -10748,7 +10642,7 @@
         <v>58.92</v>
       </c>
       <c r="AQ65" t="n">
-        <v>56.28</v>
+        <v>56.51</v>
       </c>
       <c r="AR65" t="n">
         <v>278.44</v>
@@ -10906,7 +10800,7 @@
         <v>53.6</v>
       </c>
       <c r="AQ66" t="n">
-        <v>52.66</v>
+        <v>52.5</v>
       </c>
       <c r="AR66" t="n">
         <v>145.02</v>
@@ -11064,7 +10958,7 @@
         <v>54.07</v>
       </c>
       <c r="AQ67" t="n">
-        <v>44.1</v>
+        <v>43.85</v>
       </c>
       <c r="AR67" t="n">
         <v>715.5700000000001</v>
@@ -11222,7 +11116,7 @@
         <v>35.94</v>
       </c>
       <c r="AQ68" t="n">
-        <v>36.69</v>
+        <v>36.79</v>
       </c>
       <c r="AR68" t="n">
         <v>4225.22</v>
@@ -11380,7 +11274,7 @@
         <v>55.85</v>
       </c>
       <c r="AQ69" t="n">
-        <v>47.04</v>
+        <v>45.8</v>
       </c>
       <c r="AR69" t="n">
         <v>1551.96</v>
@@ -11538,7 +11432,7 @@
         <v>64.2</v>
       </c>
       <c r="AQ70" t="n">
-        <v>53.45</v>
+        <v>52.86</v>
       </c>
       <c r="AR70" t="n">
         <v>1338.18</v>
@@ -11696,7 +11590,7 @@
         <v>41.28</v>
       </c>
       <c r="AQ71" t="n">
-        <v>43.49</v>
+        <v>43.92</v>
       </c>
       <c r="AR71" t="n">
         <v>416.34</v>
@@ -11854,7 +11748,7 @@
         <v>67.19</v>
       </c>
       <c r="AQ72" t="n">
-        <v>77.02</v>
+        <v>77.12</v>
       </c>
       <c r="AR72" t="n">
         <v>240.38</v>
@@ -12012,7 +11906,7 @@
         <v>45.61</v>
       </c>
       <c r="AQ73" t="n">
-        <v>49.69</v>
+        <v>49.32</v>
       </c>
       <c r="AR73" t="n">
         <v>1758.27</v>
@@ -12170,7 +12064,7 @@
         <v>59.92</v>
       </c>
       <c r="AQ74" t="n">
-        <v>62</v>
+        <v>61.9</v>
       </c>
       <c r="AR74" t="n">
         <v>530.89</v>
@@ -12328,7 +12222,7 @@
         <v>73.78</v>
       </c>
       <c r="AQ75" t="n">
-        <v>74.27</v>
+        <v>74.26000000000001</v>
       </c>
       <c r="AR75" t="n">
         <v>2077.6</v>
@@ -12486,7 +12380,7 @@
         <v>48.56</v>
       </c>
       <c r="AQ76" t="n">
-        <v>46.38</v>
+        <v>46.3</v>
       </c>
       <c r="AR76" t="n">
         <v>1870.12</v>
@@ -12644,7 +12538,7 @@
         <v>46.91</v>
       </c>
       <c r="AQ77" t="n">
-        <v>37.52</v>
+        <v>37.24</v>
       </c>
       <c r="AR77" t="n">
         <v>1480.22</v>
@@ -12802,7 +12696,7 @@
         <v>54.57</v>
       </c>
       <c r="AQ78" t="n">
-        <v>67.16</v>
+        <v>66.92</v>
       </c>
       <c r="AR78" t="n">
         <v>400.4</v>
@@ -12960,7 +12854,7 @@
         <v>37.3</v>
       </c>
       <c r="AQ79" t="n">
-        <v>41.8</v>
+        <v>41.61</v>
       </c>
       <c r="AR79" t="n">
         <v>656.3200000000001</v>
@@ -13118,7 +13012,7 @@
         <v>49.75</v>
       </c>
       <c r="AQ80" t="n">
-        <v>61.54</v>
+        <v>61.48</v>
       </c>
       <c r="AR80" t="n">
         <v>417.98</v>
@@ -13276,7 +13170,7 @@
         <v>42.28</v>
       </c>
       <c r="AQ81" t="n">
-        <v>43.7</v>
+        <v>43.43</v>
       </c>
       <c r="AR81" t="n">
         <v>262.4</v>
@@ -13434,7 +13328,7 @@
         <v>60.3</v>
       </c>
       <c r="AQ82" t="n">
-        <v>43.24</v>
+        <v>43.44</v>
       </c>
       <c r="AR82" t="n">
         <v>4928.51</v>
@@ -13592,7 +13486,7 @@
         <v>68.14</v>
       </c>
       <c r="AQ83" t="n">
-        <v>64.15000000000001</v>
+        <v>63.77</v>
       </c>
       <c r="AR83" t="n">
         <v>511.94</v>
@@ -13750,7 +13644,7 @@
         <v>49.44</v>
       </c>
       <c r="AQ84" t="n">
-        <v>43.25</v>
+        <v>43.13</v>
       </c>
       <c r="AR84" t="n">
         <v>1646.85</v>
@@ -13908,7 +13802,7 @@
         <v>74.04000000000001</v>
       </c>
       <c r="AQ85" t="n">
-        <v>65.25</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="AR85" t="n">
         <v>39789.95</v>
@@ -14066,7 +13960,7 @@
         <v>55.44</v>
       </c>
       <c r="AQ86" t="n">
-        <v>48.54</v>
+        <v>48.62</v>
       </c>
       <c r="AR86" t="n">
         <v>308.95</v>
@@ -14224,7 +14118,7 @@
         <v>50.98</v>
       </c>
       <c r="AQ87" t="n">
-        <v>44.09</v>
+        <v>44.13</v>
       </c>
       <c r="AR87" t="n">
         <v>530.59</v>
@@ -14382,7 +14276,7 @@
         <v>50.65</v>
       </c>
       <c r="AQ88" t="n">
-        <v>34.08</v>
+        <v>33.93</v>
       </c>
       <c r="AR88" t="n">
         <v>5222.57</v>
@@ -14540,7 +14434,7 @@
         <v>40.75</v>
       </c>
       <c r="AQ89" t="n">
-        <v>62.94</v>
+        <v>63.06</v>
       </c>
       <c r="AR89" t="n">
         <v>3964.04</v>
@@ -14698,7 +14592,7 @@
         <v>30.6</v>
       </c>
       <c r="AQ90" t="n">
-        <v>34.16</v>
+        <v>34.37</v>
       </c>
       <c r="AR90" t="n">
         <v>313.78</v>
@@ -14856,7 +14750,7 @@
         <v>54.69</v>
       </c>
       <c r="AQ91" t="n">
-        <v>57.49</v>
+        <v>57.97</v>
       </c>
       <c r="AR91" t="n">
         <v>799.4400000000001</v>
@@ -15014,7 +14908,7 @@
         <v>45.47</v>
       </c>
       <c r="AQ92" t="n">
-        <v>46.08</v>
+        <v>46.38</v>
       </c>
       <c r="AR92" t="n">
         <v>131.35</v>
@@ -15172,7 +15066,7 @@
         <v>67.33</v>
       </c>
       <c r="AQ93" t="n">
-        <v>55.91</v>
+        <v>55.87</v>
       </c>
       <c r="AR93" t="n">
         <v>878.3200000000001</v>
@@ -15330,7 +15224,7 @@
         <v>37.88</v>
       </c>
       <c r="AQ94" t="n">
-        <v>43.26</v>
+        <v>43.1</v>
       </c>
       <c r="AR94" t="n">
         <v>138.52</v>
@@ -15488,7 +15382,7 @@
         <v>74</v>
       </c>
       <c r="AQ95" t="n">
-        <v>85.01000000000001</v>
+        <v>84.92</v>
       </c>
       <c r="AR95" t="n">
         <v>2441.1</v>
@@ -15646,7 +15540,7 @@
         <v>57.04</v>
       </c>
       <c r="AQ96" t="n">
-        <v>65.73</v>
+        <v>65.17</v>
       </c>
       <c r="AR96" t="n">
         <v>1151.93</v>
@@ -15804,7 +15698,7 @@
         <v>77.59999999999999</v>
       </c>
       <c r="AQ97" t="n">
-        <v>68.72</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AR97" t="n">
         <v>2541.02</v>
@@ -15962,7 +15856,7 @@
         <v>54.08</v>
       </c>
       <c r="AQ98" t="n">
-        <v>56.71</v>
+        <v>56.52</v>
       </c>
       <c r="AR98" t="n">
         <v>185.51</v>
@@ -16120,7 +16014,7 @@
         <v>60.7</v>
       </c>
       <c r="AQ99" t="n">
-        <v>68.52</v>
+        <v>68.67</v>
       </c>
       <c r="AR99" t="n">
         <v>1147.34</v>
@@ -16436,7 +16330,7 @@
         <v>62.26</v>
       </c>
       <c r="AQ101" t="n">
-        <v>50.46</v>
+        <v>49.96</v>
       </c>
       <c r="AR101" t="n">
         <v>3440.91</v>
@@ -16594,7 +16488,7 @@
         <v>61.53</v>
       </c>
       <c r="AQ102" t="n">
-        <v>77.94</v>
+        <v>78.61</v>
       </c>
       <c r="AR102" t="n">
         <v>1205.6</v>
@@ -16752,7 +16646,7 @@
         <v>50.43</v>
       </c>
       <c r="AQ103" t="n">
-        <v>41.75</v>
+        <v>41.83</v>
       </c>
       <c r="AR103" t="n">
         <v>32.35</v>
@@ -16910,7 +16804,7 @@
         <v>39.47</v>
       </c>
       <c r="AQ104" t="n">
-        <v>48.04</v>
+        <v>47.93</v>
       </c>
       <c r="AR104" t="n">
         <v>170.49</v>
@@ -17068,7 +16962,7 @@
         <v>66.68000000000001</v>
       </c>
       <c r="AQ105" t="n">
-        <v>70.31</v>
+        <v>70.37</v>
       </c>
       <c r="AR105" t="n">
         <v>215.74</v>
@@ -17226,7 +17120,7 @@
         <v>56.22</v>
       </c>
       <c r="AQ106" t="n">
-        <v>70.29000000000001</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="AR106" t="n">
         <v>940.7</v>
@@ -17384,7 +17278,7 @@
         <v>62.82</v>
       </c>
       <c r="AQ107" t="n">
-        <v>54.61</v>
+        <v>53.64</v>
       </c>
       <c r="AR107" t="n">
         <v>799.64</v>
@@ -17542,7 +17436,7 @@
         <v>47.48</v>
       </c>
       <c r="AQ108" t="n">
-        <v>56.24</v>
+        <v>56.29</v>
       </c>
       <c r="AR108" t="n">
         <v>477.3</v>
@@ -17700,7 +17594,7 @@
         <v>45.18</v>
       </c>
       <c r="AQ109" t="n">
-        <v>56.75</v>
+        <v>56.97</v>
       </c>
       <c r="AR109" t="n">
         <v>1127.33</v>
@@ -17858,7 +17752,7 @@
         <v>64.79000000000001</v>
       </c>
       <c r="AQ110" t="n">
-        <v>54.07</v>
+        <v>53.89</v>
       </c>
       <c r="AR110" t="n">
         <v>708.65</v>
@@ -18016,7 +17910,7 @@
         <v>78.68000000000001</v>
       </c>
       <c r="AQ111" t="n">
-        <v>64.69</v>
+        <v>64.73</v>
       </c>
       <c r="AR111" t="n">
         <v>1708.72</v>
@@ -18174,7 +18068,7 @@
         <v>67.48</v>
       </c>
       <c r="AQ112" t="n">
-        <v>52.55</v>
+        <v>52.69</v>
       </c>
       <c r="AR112" t="n">
         <v>1594.16</v>
@@ -18332,7 +18226,7 @@
         <v>59.56</v>
       </c>
       <c r="AQ113" t="n">
-        <v>58.72</v>
+        <v>59.57</v>
       </c>
       <c r="AR113" t="n">
         <v>464.85</v>
@@ -18490,7 +18384,7 @@
         <v>68.93000000000001</v>
       </c>
       <c r="AQ114" t="n">
-        <v>63.54</v>
+        <v>63.44</v>
       </c>
       <c r="AR114" t="n">
         <v>1406.59</v>
@@ -18648,7 +18542,7 @@
         <v>48.47</v>
       </c>
       <c r="AQ115" t="n">
-        <v>47.67</v>
+        <v>47.63</v>
       </c>
       <c r="AR115" t="n">
         <v>787.3</v>
@@ -18806,7 +18700,7 @@
         <v>30.82</v>
       </c>
       <c r="AQ116" t="n">
-        <v>47.07</v>
+        <v>47.15</v>
       </c>
       <c r="AR116" t="n">
         <v>446.34</v>
@@ -18964,7 +18858,7 @@
         <v>47.12</v>
       </c>
       <c r="AQ117" t="n">
-        <v>44.4</v>
+        <v>44.19</v>
       </c>
       <c r="AR117" t="n">
         <v>1464.95</v>
@@ -19122,7 +19016,7 @@
         <v>62.98</v>
       </c>
       <c r="AQ118" t="n">
-        <v>57.42</v>
+        <v>57.39</v>
       </c>
       <c r="AR118" t="n">
         <v>1470.8</v>
@@ -19280,7 +19174,7 @@
         <v>64.23</v>
       </c>
       <c r="AQ119" t="n">
-        <v>56.59</v>
+        <v>56.36</v>
       </c>
       <c r="AR119" t="n">
         <v>438.23</v>
@@ -19438,7 +19332,7 @@
         <v>42.91</v>
       </c>
       <c r="AQ120" t="n">
-        <v>45.11</v>
+        <v>44.92</v>
       </c>
       <c r="AR120" t="n">
         <v>2003.46</v>
@@ -19596,7 +19490,7 @@
         <v>50.31</v>
       </c>
       <c r="AQ121" t="n">
-        <v>44.66</v>
+        <v>44.51</v>
       </c>
       <c r="AR121" t="n">
         <v>469.01</v>
@@ -19754,7 +19648,7 @@
         <v>52.49</v>
       </c>
       <c r="AQ122" t="n">
-        <v>56.2</v>
+        <v>56.1</v>
       </c>
       <c r="AR122" t="n">
         <v>1309.58</v>
@@ -19912,7 +19806,7 @@
         <v>59.67</v>
       </c>
       <c r="AQ123" t="n">
-        <v>50.69</v>
+        <v>50.66</v>
       </c>
       <c r="AR123" t="n">
         <v>1983.16</v>
@@ -20070,7 +19964,7 @@
         <v>67.22</v>
       </c>
       <c r="AQ124" t="n">
-        <v>82.86</v>
+        <v>83.09</v>
       </c>
       <c r="AR124" t="n">
         <v>3521.74</v>
@@ -20386,7 +20280,7 @@
         <v>68.63</v>
       </c>
       <c r="AQ126" t="n">
-        <v>63.37</v>
+        <v>63.04</v>
       </c>
       <c r="AR126" t="n">
         <v>1406.61</v>
@@ -20702,7 +20596,7 @@
         <v>54.32</v>
       </c>
       <c r="AQ128" t="n">
-        <v>54.11</v>
+        <v>53.82</v>
       </c>
       <c r="AR128" t="n">
         <v>272.7</v>
@@ -20860,7 +20754,7 @@
         <v>54.35</v>
       </c>
       <c r="AQ129" t="n">
-        <v>53.18</v>
+        <v>53.96</v>
       </c>
       <c r="AR129" t="n">
         <v>198.81</v>
@@ -21018,7 +20912,7 @@
         <v>48.36</v>
       </c>
       <c r="AQ130" t="n">
-        <v>64.09999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AR130" t="n">
         <v>5701.91</v>
@@ -21176,7 +21070,7 @@
         <v>50.81</v>
       </c>
       <c r="AQ131" t="n">
-        <v>44.35</v>
+        <v>44.17</v>
       </c>
       <c r="AR131" t="n">
         <v>882.53</v>
@@ -21334,7 +21228,7 @@
         <v>42.87</v>
       </c>
       <c r="AQ132" t="n">
-        <v>37.51</v>
+        <v>37.34</v>
       </c>
       <c r="AR132" t="n">
         <v>424.86</v>
@@ -21492,7 +21386,7 @@
         <v>51.02</v>
       </c>
       <c r="AQ133" t="n">
-        <v>38.66</v>
+        <v>38.33</v>
       </c>
       <c r="AR133" t="n">
         <v>1707.4</v>
@@ -21650,7 +21544,7 @@
         <v>51.97</v>
       </c>
       <c r="AQ134" t="n">
-        <v>68.59999999999999</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="AR134" t="n">
         <v>4627.82</v>
@@ -21808,7 +21702,7 @@
         <v>46.47</v>
       </c>
       <c r="AQ135" t="n">
-        <v>39.99</v>
+        <v>39.11</v>
       </c>
       <c r="AR135" t="n">
         <v>1041.77</v>
@@ -21966,7 +21860,7 @@
         <v>60.99</v>
       </c>
       <c r="AQ136" t="n">
-        <v>74.63</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="AR136" t="n">
         <v>1559.42</v>
@@ -22124,7 +22018,7 @@
         <v>40.95</v>
       </c>
       <c r="AQ137" t="n">
-        <v>48.07</v>
+        <v>47.68</v>
       </c>
       <c r="AR137" t="n">
         <v>1645.58</v>
@@ -22282,7 +22176,7 @@
         <v>54.56</v>
       </c>
       <c r="AQ138" t="n">
-        <v>57.28</v>
+        <v>57.31</v>
       </c>
       <c r="AR138" t="n">
         <v>465.14</v>
@@ -22440,7 +22334,7 @@
         <v>46.4</v>
       </c>
       <c r="AQ139" t="n">
-        <v>45.16</v>
+        <v>44.98</v>
       </c>
       <c r="AR139" t="n">
         <v>114.4</v>
@@ -22598,7 +22492,7 @@
         <v>51.59</v>
       </c>
       <c r="AQ140" t="n">
-        <v>59.59</v>
+        <v>58.91</v>
       </c>
       <c r="AR140" t="n">
         <v>6722.45</v>
@@ -22756,7 +22650,7 @@
         <v>52.83</v>
       </c>
       <c r="AQ141" t="n">
-        <v>55.52</v>
+        <v>55.73</v>
       </c>
       <c r="AR141" t="n">
         <v>12109.89</v>
@@ -22914,7 +22808,7 @@
         <v>58.34</v>
       </c>
       <c r="AQ142" t="n">
-        <v>54.6</v>
+        <v>54.78</v>
       </c>
       <c r="AR142" t="n">
         <v>615.9400000000001</v>
@@ -23072,7 +22966,7 @@
         <v>57.2</v>
       </c>
       <c r="AQ143" t="n">
-        <v>55.45</v>
+        <v>55.6</v>
       </c>
       <c r="AR143" t="n">
         <v>4275.3</v>
@@ -23230,7 +23124,7 @@
         <v>49.92</v>
       </c>
       <c r="AQ144" t="n">
-        <v>46.44</v>
+        <v>45.99</v>
       </c>
       <c r="AR144" t="n">
         <v>2273.44</v>
@@ -23388,7 +23282,7 @@
         <v>75.45999999999999</v>
       </c>
       <c r="AQ145" t="n">
-        <v>62.89</v>
+        <v>62.76</v>
       </c>
       <c r="AR145" t="n">
         <v>1303.25</v>
@@ -23546,7 +23440,7 @@
         <v>45.03</v>
       </c>
       <c r="AQ146" t="n">
-        <v>37.9</v>
+        <v>37.72</v>
       </c>
       <c r="AR146" t="n">
         <v>1413.25</v>
@@ -23704,7 +23598,7 @@
         <v>64.43000000000001</v>
       </c>
       <c r="AQ147" t="n">
-        <v>58.96</v>
+        <v>59.01</v>
       </c>
       <c r="AR147" t="n">
         <v>7536.83</v>
@@ -23862,7 +23756,7 @@
         <v>36.93</v>
       </c>
       <c r="AQ148" t="n">
-        <v>21.86</v>
+        <v>21.57</v>
       </c>
       <c r="AR148" t="n">
         <v>716.85</v>
@@ -24020,7 +23914,7 @@
         <v>66</v>
       </c>
       <c r="AQ149" t="n">
-        <v>52.62</v>
+        <v>52.64</v>
       </c>
       <c r="AR149" t="n">
         <v>319.49</v>
@@ -24178,7 +24072,7 @@
         <v>45.82</v>
       </c>
       <c r="AQ150" t="n">
-        <v>56.96</v>
+        <v>57.68</v>
       </c>
       <c r="AR150" t="n">
         <v>535.64</v>
@@ -24336,7 +24230,7 @@
         <v>54.44</v>
       </c>
       <c r="AQ151" t="n">
-        <v>66.45</v>
+        <v>66.31</v>
       </c>
       <c r="AR151" t="n">
         <v>607.52</v>
@@ -24494,7 +24388,7 @@
         <v>44.72</v>
       </c>
       <c r="AQ152" t="n">
-        <v>38.61</v>
+        <v>38.42</v>
       </c>
       <c r="AR152" t="n">
         <v>400.82</v>
@@ -24652,7 +24546,7 @@
         <v>72.98</v>
       </c>
       <c r="AQ153" t="n">
-        <v>74.52</v>
+        <v>74.75</v>
       </c>
       <c r="AR153" t="n">
         <v>1798.42</v>
@@ -24810,7 +24704,7 @@
         <v>60.17</v>
       </c>
       <c r="AQ154" t="n">
-        <v>76.04000000000001</v>
+        <v>76.09</v>
       </c>
       <c r="AR154" t="n">
         <v>333.37</v>
@@ -24968,7 +24862,7 @@
         <v>62.97</v>
       </c>
       <c r="AQ155" t="n">
-        <v>59.39</v>
+        <v>59.51</v>
       </c>
       <c r="AR155" t="n">
         <v>2653.44</v>
@@ -25126,7 +25020,7 @@
         <v>57.79</v>
       </c>
       <c r="AQ156" t="n">
-        <v>62.95</v>
+        <v>62.97</v>
       </c>
       <c r="AR156" t="n">
         <v>249.55</v>
@@ -25284,7 +25178,7 @@
         <v>53.06</v>
       </c>
       <c r="AQ157" t="n">
-        <v>63.3</v>
+        <v>63.09</v>
       </c>
       <c r="AR157" t="n">
         <v>3721.97</v>
@@ -25442,7 +25336,7 @@
         <v>64.48999999999999</v>
       </c>
       <c r="AQ158" t="n">
-        <v>58.06</v>
+        <v>58.14</v>
       </c>
       <c r="AR158" t="n">
         <v>1435.75</v>
@@ -25600,7 +25494,7 @@
         <v>62.59</v>
       </c>
       <c r="AQ159" t="n">
-        <v>42.03</v>
+        <v>41.88</v>
       </c>
       <c r="AR159" t="n">
         <v>2887.78</v>
@@ -25758,7 +25652,7 @@
         <v>52.51</v>
       </c>
       <c r="AQ160" t="n">
-        <v>49.73</v>
+        <v>49.66</v>
       </c>
       <c r="AR160" t="n">
         <v>256.31</v>
@@ -25916,7 +25810,7 @@
         <v>54.35</v>
       </c>
       <c r="AQ161" t="n">
-        <v>63.29</v>
+        <v>63.35</v>
       </c>
       <c r="AR161" t="n">
         <v>388.02</v>
@@ -26074,7 +25968,7 @@
         <v>46.85</v>
       </c>
       <c r="AQ162" t="n">
-        <v>55.89</v>
+        <v>55.71</v>
       </c>
       <c r="AR162" t="n">
         <v>906.03</v>
@@ -26232,7 +26126,7 @@
         <v>69.39</v>
       </c>
       <c r="AQ163" t="n">
-        <v>71.47</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="AR163" t="n">
         <v>320.59</v>
@@ -26390,7 +26284,7 @@
         <v>54.51</v>
       </c>
       <c r="AQ164" t="n">
-        <v>61.24</v>
+        <v>61.29</v>
       </c>
       <c r="AR164" t="n">
         <v>1122.69</v>
@@ -26548,7 +26442,7 @@
         <v>51.71</v>
       </c>
       <c r="AQ165" t="n">
-        <v>39.83</v>
+        <v>39.25</v>
       </c>
       <c r="AR165" t="n">
         <v>220.73</v>
@@ -26706,7 +26600,7 @@
         <v>63.23</v>
       </c>
       <c r="AQ166" t="n">
-        <v>56.85</v>
+        <v>56.61</v>
       </c>
       <c r="AR166" t="n">
         <v>488.86</v>
@@ -26864,7 +26758,7 @@
         <v>73.13</v>
       </c>
       <c r="AQ167" t="n">
-        <v>64.38</v>
+        <v>63.55</v>
       </c>
       <c r="AR167" t="n">
         <v>3823.53</v>
@@ -27022,7 +26916,7 @@
         <v>48.71</v>
       </c>
       <c r="AQ168" t="n">
-        <v>41.64</v>
+        <v>41.68</v>
       </c>
       <c r="AR168" t="n">
         <v>18278.99</v>
@@ -27180,7 +27074,7 @@
         <v>44.57</v>
       </c>
       <c r="AQ169" t="n">
-        <v>55.51</v>
+        <v>55.23</v>
       </c>
       <c r="AR169" t="n">
         <v>967.4</v>
@@ -27338,7 +27232,7 @@
         <v>42.68</v>
       </c>
       <c r="AQ170" t="n">
-        <v>45.99</v>
+        <v>45.57</v>
       </c>
       <c r="AR170" t="n">
         <v>244.95</v>
@@ -27496,7 +27390,7 @@
         <v>66.75</v>
       </c>
       <c r="AQ171" t="n">
-        <v>65.27</v>
+        <v>64.87</v>
       </c>
       <c r="AR171" t="n">
         <v>1184.37</v>
@@ -27654,7 +27548,7 @@
         <v>54.53</v>
       </c>
       <c r="AQ172" t="n">
-        <v>61.86</v>
+        <v>61.95</v>
       </c>
       <c r="AR172" t="n">
         <v>173.69</v>
@@ -27812,7 +27706,7 @@
         <v>53.37</v>
       </c>
       <c r="AQ173" t="n">
-        <v>55.45</v>
+        <v>55.35</v>
       </c>
       <c r="AR173" t="n">
         <v>709.6900000000001</v>
@@ -27970,7 +27864,7 @@
         <v>56.91</v>
       </c>
       <c r="AQ174" t="n">
-        <v>57.09</v>
+        <v>57.15</v>
       </c>
       <c r="AR174" t="n">
         <v>1460.79</v>
@@ -28128,7 +28022,7 @@
         <v>39.82</v>
       </c>
       <c r="AQ175" t="n">
-        <v>37.96</v>
+        <v>38.03</v>
       </c>
       <c r="AR175" t="n">
         <v>366.66</v>
@@ -28286,7 +28180,7 @@
         <v>43.3</v>
       </c>
       <c r="AQ176" t="n">
-        <v>43.04</v>
+        <v>42.77</v>
       </c>
       <c r="AR176" t="n">
         <v>7786.24</v>
@@ -28444,7 +28338,7 @@
         <v>62.68</v>
       </c>
       <c r="AQ177" t="n">
-        <v>70</v>
+        <v>69.93000000000001</v>
       </c>
       <c r="AR177" t="n">
         <v>2262.99</v>
@@ -28602,7 +28496,7 @@
         <v>65.14</v>
       </c>
       <c r="AQ178" t="n">
-        <v>52.21</v>
+        <v>52.87</v>
       </c>
       <c r="AR178" t="n">
         <v>2307.39</v>
@@ -28760,7 +28654,7 @@
         <v>41.15</v>
       </c>
       <c r="AQ179" t="n">
-        <v>47.66</v>
+        <v>47.27</v>
       </c>
       <c r="AR179" t="n">
         <v>2174.23</v>
@@ -28918,7 +28812,7 @@
         <v>32.58</v>
       </c>
       <c r="AQ180" t="n">
-        <v>44.17</v>
+        <v>43.86</v>
       </c>
       <c r="AR180" t="n">
         <v>606.64</v>
@@ -29076,7 +28970,7 @@
         <v>64.65000000000001</v>
       </c>
       <c r="AQ181" t="n">
-        <v>66.04000000000001</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="AR181" t="n">
         <v>107.33</v>
@@ -29234,7 +29128,7 @@
         <v>48.02</v>
       </c>
       <c r="AQ182" t="n">
-        <v>48.15</v>
+        <v>47.7</v>
       </c>
       <c r="AR182" t="n">
         <v>2253.97</v>
@@ -29392,7 +29286,7 @@
         <v>57.96</v>
       </c>
       <c r="AQ183" t="n">
-        <v>44.06</v>
+        <v>44.47</v>
       </c>
       <c r="AR183" t="n">
         <v>309.23</v>
@@ -29550,7 +29444,7 @@
         <v>56.54</v>
       </c>
       <c r="AQ184" t="n">
-        <v>44.97</v>
+        <v>45.28</v>
       </c>
       <c r="AR184" t="n">
         <v>1021.31</v>
@@ -29708,7 +29602,7 @@
         <v>68.87</v>
       </c>
       <c r="AQ185" t="n">
-        <v>62.04</v>
+        <v>62.66</v>
       </c>
       <c r="AR185" t="n">
         <v>1115.62</v>
@@ -29866,7 +29760,7 @@
         <v>66.51000000000001</v>
       </c>
       <c r="AQ186" t="n">
-        <v>55.83</v>
+        <v>55.8</v>
       </c>
       <c r="AR186" t="n">
         <v>1794.31</v>
@@ -30024,7 +29918,7 @@
         <v>34.78</v>
       </c>
       <c r="AQ187" t="n">
-        <v>42.17</v>
+        <v>42.39</v>
       </c>
       <c r="AR187" t="n">
         <v>271.47</v>
@@ -30182,7 +30076,7 @@
         <v>48.93</v>
       </c>
       <c r="AQ188" t="n">
-        <v>67.41</v>
+        <v>67.66</v>
       </c>
       <c r="AR188" t="n">
         <v>771.13</v>
@@ -30340,7 +30234,7 @@
         <v>25.31</v>
       </c>
       <c r="AQ189" t="n">
-        <v>38.35</v>
+        <v>38.23</v>
       </c>
       <c r="AR189" t="n">
         <v>636.1799999999999</v>
@@ -30498,7 +30392,7 @@
         <v>54.27</v>
       </c>
       <c r="AQ190" t="n">
-        <v>66.5</v>
+        <v>66.84</v>
       </c>
       <c r="AR190" t="n">
         <v>3135.53</v>
@@ -30656,7 +30550,7 @@
         <v>51.13</v>
       </c>
       <c r="AQ191" t="n">
-        <v>53.54</v>
+        <v>53.84</v>
       </c>
       <c r="AR191" t="n">
         <v>1687.42</v>
@@ -30814,7 +30708,7 @@
         <v>55.37</v>
       </c>
       <c r="AQ192" t="n">
-        <v>61.61</v>
+        <v>61.43</v>
       </c>
       <c r="AR192" t="n">
         <v>198.21</v>
@@ -30972,7 +30866,7 @@
         <v>49.96</v>
       </c>
       <c r="AQ193" t="n">
-        <v>54.37</v>
+        <v>54.15</v>
       </c>
       <c r="AR193" t="n">
         <v>2757.61</v>
@@ -31130,7 +31024,7 @@
         <v>50.42</v>
       </c>
       <c r="AQ194" t="n">
-        <v>63.06</v>
+        <v>63.22</v>
       </c>
       <c r="AR194" t="n">
         <v>5159.82</v>
@@ -31288,7 +31182,7 @@
         <v>51.09</v>
       </c>
       <c r="AQ195" t="n">
-        <v>53.36</v>
+        <v>53.2</v>
       </c>
       <c r="AR195" t="n">
         <v>4385.86</v>
@@ -31446,7 +31340,7 @@
         <v>49.77</v>
       </c>
       <c r="AQ196" t="n">
-        <v>36.93</v>
+        <v>37.04</v>
       </c>
       <c r="AR196" t="n">
         <v>1177.95</v>
@@ -31604,7 +31498,7 @@
         <v>63.38</v>
       </c>
       <c r="AQ197" t="n">
-        <v>55.97</v>
+        <v>55.8</v>
       </c>
       <c r="AR197" t="n">
         <v>811.26</v>
@@ -31762,7 +31656,7 @@
         <v>34.94</v>
       </c>
       <c r="AQ198" t="n">
-        <v>28.54</v>
+        <v>28.53</v>
       </c>
       <c r="AR198" t="n">
         <v>1125.59</v>
@@ -31920,7 +31814,7 @@
         <v>75.65000000000001</v>
       </c>
       <c r="AQ199" t="n">
-        <v>62.19</v>
+        <v>61.98</v>
       </c>
       <c r="AR199" t="n">
         <v>712.6799999999999</v>
@@ -32078,7 +31972,7 @@
         <v>54.21</v>
       </c>
       <c r="AQ200" t="n">
-        <v>53.21</v>
+        <v>53.37</v>
       </c>
       <c r="AR200" t="n">
         <v>2644.26</v>
@@ -32236,7 +32130,7 @@
         <v>67.81999999999999</v>
       </c>
       <c r="AQ201" t="n">
-        <v>49.07</v>
+        <v>48.99</v>
       </c>
       <c r="AR201" t="n">
         <v>779.22</v>
@@ -32394,7 +32288,7 @@
         <v>50.95</v>
       </c>
       <c r="AQ202" t="n">
-        <v>40.56</v>
+        <v>40.43</v>
       </c>
       <c r="AR202" t="n">
         <v>585.85</v>
@@ -32552,7 +32446,7 @@
         <v>33.92</v>
       </c>
       <c r="AQ203" t="n">
-        <v>41.2</v>
+        <v>41.19</v>
       </c>
       <c r="AR203" t="n">
         <v>531.41</v>
@@ -32710,7 +32604,7 @@
         <v>42.68</v>
       </c>
       <c r="AQ204" t="n">
-        <v>41.25</v>
+        <v>41.58</v>
       </c>
       <c r="AR204" t="n">
         <v>4944.42</v>
@@ -32868,7 +32762,7 @@
         <v>44.92</v>
       </c>
       <c r="AQ205" t="n">
-        <v>44.52</v>
+        <v>44.81</v>
       </c>
       <c r="AR205" t="n">
         <v>497.56</v>
@@ -33184,7 +33078,7 @@
         <v>26.46</v>
       </c>
       <c r="AQ207" t="n">
-        <v>43.5</v>
+        <v>43.35</v>
       </c>
       <c r="AR207" t="n">
         <v>996.97</v>
@@ -33342,7 +33236,7 @@
         <v>31.54</v>
       </c>
       <c r="AQ208" t="n">
-        <v>42.63</v>
+        <v>42.32</v>
       </c>
       <c r="AR208" t="n">
         <v>505.83</v>
@@ -33500,7 +33394,7 @@
         <v>61.55</v>
       </c>
       <c r="AQ209" t="n">
-        <v>55.11</v>
+        <v>55.03</v>
       </c>
       <c r="AR209" t="n">
         <v>399.99</v>
@@ -33658,7 +33552,7 @@
         <v>54.72</v>
       </c>
       <c r="AQ210" t="n">
-        <v>46.44</v>
+        <v>46.76</v>
       </c>
       <c r="AR210" t="n">
         <v>2161.76</v>
@@ -33816,7 +33710,7 @@
         <v>25.28</v>
       </c>
       <c r="AQ211" t="n">
-        <v>38.46</v>
+        <v>38.58</v>
       </c>
       <c r="AR211" t="n">
         <v>552.1900000000001</v>
@@ -33974,7 +33868,7 @@
         <v>67.45</v>
       </c>
       <c r="AQ212" t="n">
-        <v>61.77</v>
+        <v>61.8</v>
       </c>
       <c r="AR212" t="n">
         <v>1144.33</v>
@@ -34132,7 +34026,7 @@
         <v>61.68</v>
       </c>
       <c r="AQ213" t="n">
-        <v>80.17</v>
+        <v>79.83</v>
       </c>
       <c r="AR213" t="n">
         <v>413.93</v>
@@ -34290,7 +34184,7 @@
         <v>77.27</v>
       </c>
       <c r="AQ214" t="n">
-        <v>70.90000000000001</v>
+        <v>70.91</v>
       </c>
       <c r="AR214" t="n">
         <v>37825.87</v>
@@ -34448,7 +34342,7 @@
         <v>57.74</v>
       </c>
       <c r="AQ215" t="n">
-        <v>73.75</v>
+        <v>73.81</v>
       </c>
       <c r="AR215" t="n">
         <v>667.86</v>
@@ -34606,7 +34500,7 @@
         <v>49.82</v>
       </c>
       <c r="AQ216" t="n">
-        <v>53.91</v>
+        <v>53.68</v>
       </c>
       <c r="AR216" t="n">
         <v>208.97</v>
@@ -34764,7 +34658,7 @@
         <v>56.61</v>
       </c>
       <c r="AQ217" t="n">
-        <v>49.01</v>
+        <v>48.71</v>
       </c>
       <c r="AR217" t="n">
         <v>1963.84</v>
@@ -34922,7 +34816,7 @@
         <v>51.51</v>
       </c>
       <c r="AQ218" t="n">
-        <v>57.92</v>
+        <v>57.37</v>
       </c>
       <c r="AR218" t="n">
         <v>3345.75</v>
@@ -35080,7 +34974,7 @@
         <v>74.77</v>
       </c>
       <c r="AQ219" t="n">
-        <v>63.2</v>
+        <v>63.14</v>
       </c>
       <c r="AR219" t="n">
         <v>1348.82</v>
@@ -35238,7 +35132,7 @@
         <v>53.62</v>
       </c>
       <c r="AQ220" t="n">
-        <v>49.57</v>
+        <v>50.1</v>
       </c>
       <c r="AR220" t="n">
         <v>1813.21</v>
@@ -35396,7 +35290,7 @@
         <v>46.77</v>
       </c>
       <c r="AQ221" t="n">
-        <v>38.58</v>
+        <v>38.59</v>
       </c>
       <c r="AR221" t="n">
         <v>495.64</v>
@@ -35554,7 +35448,7 @@
         <v>63.88</v>
       </c>
       <c r="AQ222" t="n">
-        <v>54.7</v>
+        <v>54.27</v>
       </c>
       <c r="AR222" t="n">
         <v>83.95999999999999</v>
@@ -35712,7 +35606,7 @@
         <v>45.54</v>
       </c>
       <c r="AQ223" t="n">
-        <v>68.12</v>
+        <v>68.01000000000001</v>
       </c>
       <c r="AR223" t="n">
         <v>14.5</v>
@@ -35870,7 +35764,7 @@
         <v>69.55</v>
       </c>
       <c r="AQ224" t="n">
-        <v>62.9</v>
+        <v>63.16</v>
       </c>
       <c r="AR224" t="n">
         <v>78.17</v>
@@ -36186,7 +36080,7 @@
         <v>48.23</v>
       </c>
       <c r="AQ226" t="n">
-        <v>62.87</v>
+        <v>62.75</v>
       </c>
       <c r="AR226" t="n">
         <v>81.13</v>
@@ -36344,7 +36238,7 @@
         <v>50.47</v>
       </c>
       <c r="AQ227" t="n">
-        <v>55</v>
+        <v>55.12</v>
       </c>
       <c r="AR227" t="n">
         <v>358.2</v>
@@ -36502,7 +36396,7 @@
         <v>60.93</v>
       </c>
       <c r="AQ228" t="n">
-        <v>54.47</v>
+        <v>54.28</v>
       </c>
       <c r="AR228" t="n">
         <v>168.39</v>
@@ -36660,7 +36554,7 @@
         <v>49.71</v>
       </c>
       <c r="AQ229" t="n">
-        <v>54.21</v>
+        <v>54.05</v>
       </c>
       <c r="AR229" t="n">
         <v>522.29</v>
@@ -36818,7 +36712,7 @@
         <v>58.88</v>
       </c>
       <c r="AQ230" t="n">
-        <v>60.45</v>
+        <v>60.21</v>
       </c>
       <c r="AR230" t="n">
         <v>1687.95</v>
@@ -36976,7 +36870,7 @@
         <v>47.99</v>
       </c>
       <c r="AQ231" t="n">
-        <v>54.91</v>
+        <v>54.13</v>
       </c>
       <c r="AR231" t="n">
         <v>524.01</v>
@@ -37134,7 +37028,7 @@
         <v>69.8</v>
       </c>
       <c r="AQ232" t="n">
-        <v>65</v>
+        <v>65.39</v>
       </c>
       <c r="AR232" t="n">
         <v>710.25</v>
@@ -37292,7 +37186,7 @@
         <v>48.11</v>
       </c>
       <c r="AQ233" t="n">
-        <v>45.56</v>
+        <v>45.62</v>
       </c>
       <c r="AR233" t="n">
         <v>382.6</v>
@@ -37450,7 +37344,7 @@
         <v>42.92</v>
       </c>
       <c r="AQ234" t="n">
-        <v>41.82</v>
+        <v>42.19</v>
       </c>
       <c r="AR234" t="n">
         <v>1998.64</v>
@@ -37608,7 +37502,7 @@
         <v>45.06</v>
       </c>
       <c r="AQ235" t="n">
-        <v>47.07</v>
+        <v>47.46</v>
       </c>
       <c r="AR235" t="n">
         <v>848.45</v>
@@ -37766,7 +37660,7 @@
         <v>82.31</v>
       </c>
       <c r="AQ236" t="n">
-        <v>69.81</v>
+        <v>69.98</v>
       </c>
       <c r="AR236" t="n">
         <v>5042.67</v>
@@ -37924,7 +37818,7 @@
         <v>51.08</v>
       </c>
       <c r="AQ237" t="n">
-        <v>55.51</v>
+        <v>55.21</v>
       </c>
       <c r="AR237" t="n">
         <v>921</v>
@@ -38082,7 +37976,7 @@
         <v>26.08</v>
       </c>
       <c r="AQ238" t="n">
-        <v>38.44</v>
+        <v>38.56</v>
       </c>
       <c r="AR238" t="n">
         <v>406.38</v>
@@ -38240,7 +38134,7 @@
         <v>34.71</v>
       </c>
       <c r="AQ239" t="n">
-        <v>28.24</v>
+        <v>28.36</v>
       </c>
       <c r="AR239" t="n">
         <v>1078.73</v>
@@ -38398,7 +38292,7 @@
         <v>48.7</v>
       </c>
       <c r="AQ240" t="n">
-        <v>38.78</v>
+        <v>38.65</v>
       </c>
       <c r="AR240" t="n">
         <v>89.88</v>
@@ -38556,7 +38450,7 @@
         <v>52.09</v>
       </c>
       <c r="AQ241" t="n">
-        <v>47.57</v>
+        <v>47.66</v>
       </c>
       <c r="AR241" t="n">
         <v>750.05</v>
@@ -38714,7 +38608,7 @@
         <v>53.24</v>
       </c>
       <c r="AQ242" t="n">
-        <v>49.61</v>
+        <v>49.48</v>
       </c>
       <c r="AR242" t="n">
         <v>34.63</v>
@@ -38872,7 +38766,7 @@
         <v>53.95</v>
       </c>
       <c r="AQ243" t="n">
-        <v>46.8</v>
+        <v>46.86</v>
       </c>
       <c r="AR243" t="n">
         <v>143.72</v>
@@ -39030,7 +38924,7 @@
         <v>58.02</v>
       </c>
       <c r="AQ244" t="n">
-        <v>58.75</v>
+        <v>58.89</v>
       </c>
       <c r="AR244" t="n">
         <v>1599.4</v>
@@ -39188,7 +39082,7 @@
         <v>48.96</v>
       </c>
       <c r="AQ245" t="n">
-        <v>49.8</v>
+        <v>49.38</v>
       </c>
       <c r="AR245" t="n">
         <v>21.29</v>
@@ -39346,7 +39240,7 @@
         <v>41.39</v>
       </c>
       <c r="AQ246" t="n">
-        <v>40.74</v>
+        <v>40.46</v>
       </c>
       <c r="AR246" t="n">
         <v>136.54</v>
@@ -39504,7 +39398,7 @@
         <v>41.49</v>
       </c>
       <c r="AQ247" t="n">
-        <v>36.23</v>
+        <v>36.2</v>
       </c>
       <c r="AR247" t="n">
         <v>518.3200000000001</v>
@@ -39662,7 +39556,7 @@
         <v>52.98</v>
       </c>
       <c r="AQ248" t="n">
-        <v>48.87</v>
+        <v>48.29</v>
       </c>
       <c r="AR248" t="n">
         <v>126.94</v>
@@ -39820,7 +39714,7 @@
         <v>33.37</v>
       </c>
       <c r="AQ249" t="n">
-        <v>33.55</v>
+        <v>33.51</v>
       </c>
       <c r="AR249" t="n">
         <v>96.29000000000001</v>
@@ -40136,7 +40030,7 @@
         <v>68.89</v>
       </c>
       <c r="AQ251" t="n">
-        <v>58.68</v>
+        <v>58.92</v>
       </c>
       <c r="AR251" t="n">
         <v>169.44</v>
@@ -40294,7 +40188,7 @@
         <v>49.06</v>
       </c>
       <c r="AQ252" t="n">
-        <v>54.45</v>
+        <v>54.25</v>
       </c>
       <c r="AR252" t="n">
         <v>305.55</v>
@@ -40452,7 +40346,7 @@
         <v>60.74</v>
       </c>
       <c r="AQ253" t="n">
-        <v>71.77</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="AR253" t="n">
         <v>159.4</v>
@@ -40610,7 +40504,7 @@
         <v>41.2</v>
       </c>
       <c r="AQ254" t="n">
-        <v>41.71</v>
+        <v>41.7</v>
       </c>
       <c r="AR254" t="n">
         <v>363.84</v>
@@ -40768,7 +40662,7 @@
         <v>63.5</v>
       </c>
       <c r="AQ255" t="n">
-        <v>68.69</v>
+        <v>67.38</v>
       </c>
       <c r="AR255" t="n">
         <v>2219.44</v>
@@ -40926,7 +40820,7 @@
         <v>53.66</v>
       </c>
       <c r="AQ256" t="n">
-        <v>62.03</v>
+        <v>62.45</v>
       </c>
       <c r="AR256" t="n">
         <v>700.6799999999999</v>
@@ -41084,7 +40978,7 @@
         <v>61.88</v>
       </c>
       <c r="AQ257" t="n">
-        <v>66.94</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="AR257" t="n">
         <v>255.27</v>
@@ -41242,7 +41136,7 @@
         <v>20.74</v>
       </c>
       <c r="AQ258" t="n">
-        <v>34.01</v>
+        <v>34.15</v>
       </c>
       <c r="AR258" t="n">
         <v>1109.71</v>
@@ -41400,7 +41294,7 @@
         <v>51.08</v>
       </c>
       <c r="AQ259" t="n">
-        <v>42.15</v>
+        <v>41.85</v>
       </c>
       <c r="AR259" t="n">
         <v>239.77</v>
@@ -41558,7 +41452,7 @@
         <v>66.29000000000001</v>
       </c>
       <c r="AQ260" t="n">
-        <v>53.79</v>
+        <v>53.35</v>
       </c>
       <c r="AR260" t="n">
         <v>5417.03</v>
@@ -41716,7 +41610,7 @@
         <v>53.63</v>
       </c>
       <c r="AQ261" t="n">
-        <v>44.69</v>
+        <v>44.71</v>
       </c>
       <c r="AR261" t="n">
         <v>397.16</v>
@@ -41874,7 +41768,7 @@
         <v>52.2</v>
       </c>
       <c r="AQ262" t="n">
-        <v>45.99</v>
+        <v>45.7</v>
       </c>
       <c r="AR262" t="n">
         <v>125.22</v>
@@ -42032,7 +41926,7 @@
         <v>41.97</v>
       </c>
       <c r="AQ263" t="n">
-        <v>49.75</v>
+        <v>49.47</v>
       </c>
       <c r="AR263" t="n">
         <v>18.13</v>
@@ -42190,7 +42084,7 @@
         <v>46.46</v>
       </c>
       <c r="AQ264" t="n">
-        <v>38.02</v>
+        <v>37.81</v>
       </c>
       <c r="AR264" t="n">
         <v>698.0599999999999</v>
@@ -42348,7 +42242,7 @@
         <v>62.92</v>
       </c>
       <c r="AQ265" t="n">
-        <v>60.15</v>
+        <v>59.86</v>
       </c>
       <c r="AR265" t="n">
         <v>130.75</v>
@@ -42506,7 +42400,7 @@
         <v>54.75</v>
       </c>
       <c r="AQ266" t="n">
-        <v>59</v>
+        <v>59.06</v>
       </c>
       <c r="AR266" t="n">
         <v>3216.08</v>
@@ -42664,7 +42558,7 @@
         <v>52.96</v>
       </c>
       <c r="AQ267" t="n">
-        <v>59.72</v>
+        <v>59.66</v>
       </c>
       <c r="AR267" t="n">
         <v>572.14</v>
@@ -42822,7 +42716,7 @@
         <v>74.06999999999999</v>
       </c>
       <c r="AQ268" t="n">
-        <v>76.23</v>
+        <v>76.37</v>
       </c>
       <c r="AR268" t="n">
         <v>312.41</v>
@@ -42980,7 +42874,7 @@
         <v>32.54</v>
       </c>
       <c r="AQ269" t="n">
-        <v>47.88</v>
+        <v>47.93</v>
       </c>
       <c r="AR269" t="n">
         <v>1260.65</v>
@@ -43138,7 +43032,7 @@
         <v>45.45</v>
       </c>
       <c r="AQ270" t="n">
-        <v>30.33</v>
+        <v>30.69</v>
       </c>
       <c r="AR270" t="n">
         <v>424.11</v>
@@ -43296,7 +43190,7 @@
         <v>36.42</v>
       </c>
       <c r="AQ271" t="n">
-        <v>43.33</v>
+        <v>43.31</v>
       </c>
       <c r="AR271" t="n">
         <v>634.12</v>
@@ -43454,7 +43348,7 @@
         <v>46.01</v>
       </c>
       <c r="AQ272" t="n">
-        <v>50.94</v>
+        <v>50.84</v>
       </c>
       <c r="AR272" t="n">
         <v>970.59</v>
@@ -43612,7 +43506,7 @@
         <v>35.14</v>
       </c>
       <c r="AQ273" t="n">
-        <v>41.96</v>
+        <v>42.01</v>
       </c>
       <c r="AR273" t="n">
         <v>272.84</v>
@@ -43770,7 +43664,7 @@
         <v>68.45</v>
       </c>
       <c r="AQ274" t="n">
-        <v>51.77</v>
+        <v>52.28</v>
       </c>
       <c r="AR274" t="n">
         <v>727.92</v>
@@ -43928,7 +43822,7 @@
         <v>72.67</v>
       </c>
       <c r="AQ275" t="n">
-        <v>66.19</v>
+        <v>66.31999999999999</v>
       </c>
       <c r="AR275" t="n">
         <v>1167.44</v>
@@ -44086,7 +43980,7 @@
         <v>55.97</v>
       </c>
       <c r="AQ276" t="n">
-        <v>45.27</v>
+        <v>44.94</v>
       </c>
       <c r="AR276" t="n">
         <v>374.58</v>
@@ -44244,7 +44138,7 @@
         <v>49.74</v>
       </c>
       <c r="AQ277" t="n">
-        <v>52.2</v>
+        <v>51.92</v>
       </c>
       <c r="AR277" t="n">
         <v>292.26</v>
@@ -44402,7 +44296,7 @@
         <v>51.2</v>
       </c>
       <c r="AQ278" t="n">
-        <v>38.48</v>
+        <v>38.38</v>
       </c>
       <c r="AR278" t="n">
         <v>3225.55</v>
@@ -44560,7 +44454,7 @@
         <v>54.51</v>
       </c>
       <c r="AQ279" t="n">
-        <v>41.28</v>
+        <v>41.08</v>
       </c>
       <c r="AR279" t="n">
         <v>527.78</v>
@@ -44718,7 +44612,7 @@
         <v>44.06</v>
       </c>
       <c r="AQ280" t="n">
-        <v>60.6</v>
+        <v>60.37</v>
       </c>
       <c r="AR280" t="n">
         <v>5454.72</v>
@@ -44876,7 +44770,7 @@
         <v>51.61</v>
       </c>
       <c r="AQ281" t="n">
-        <v>44.62</v>
+        <v>44.83</v>
       </c>
       <c r="AR281" t="n">
         <v>880.34</v>
@@ -45034,7 +44928,7 @@
         <v>56.78</v>
       </c>
       <c r="AQ282" t="n">
-        <v>67.27</v>
+        <v>66.87</v>
       </c>
       <c r="AR282" t="n">
         <v>794.14</v>
@@ -45192,7 +45086,7 @@
         <v>78.92</v>
       </c>
       <c r="AQ283" t="n">
-        <v>86.88</v>
+        <v>86.78</v>
       </c>
       <c r="AR283" t="n">
         <v>2263.58</v>
@@ -45350,7 +45244,7 @@
         <v>69.25</v>
       </c>
       <c r="AQ284" t="n">
-        <v>59.24</v>
+        <v>59.57</v>
       </c>
       <c r="AR284" t="n">
         <v>402.5</v>
@@ -45508,7 +45402,7 @@
         <v>59.89</v>
       </c>
       <c r="AQ285" t="n">
-        <v>70.18000000000001</v>
+        <v>69.55</v>
       </c>
       <c r="AR285" t="n">
         <v>1381.49</v>
@@ -45666,7 +45560,7 @@
         <v>45.34</v>
       </c>
       <c r="AQ286" t="n">
-        <v>39.7</v>
+        <v>39.17</v>
       </c>
       <c r="AR286" t="n">
         <v>747.62</v>
@@ -45824,7 +45718,7 @@
         <v>67.2</v>
       </c>
       <c r="AQ287" t="n">
-        <v>77.29000000000001</v>
+        <v>77.76000000000001</v>
       </c>
       <c r="AR287" t="n">
         <v>1142.97</v>
@@ -45982,7 +45876,7 @@
         <v>67.56</v>
       </c>
       <c r="AQ288" t="n">
-        <v>68</v>
+        <v>68.11</v>
       </c>
       <c r="AR288" t="n">
         <v>1650.06</v>
@@ -46140,7 +46034,7 @@
         <v>45.69</v>
       </c>
       <c r="AQ289" t="n">
-        <v>39.21</v>
+        <v>39.19</v>
       </c>
       <c r="AR289" t="n">
         <v>299.4</v>
@@ -46298,7 +46192,7 @@
         <v>63.88</v>
       </c>
       <c r="AQ290" t="n">
-        <v>77.25</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="AR290" t="n">
         <v>1428.36</v>
@@ -46456,7 +46350,7 @@
         <v>67.28</v>
       </c>
       <c r="AQ291" t="n">
-        <v>51.08</v>
+        <v>50.53</v>
       </c>
       <c r="AR291" t="n">
         <v>115.56</v>
@@ -46614,7 +46508,7 @@
         <v>50.79</v>
       </c>
       <c r="AQ292" t="n">
-        <v>53.03</v>
+        <v>52.7</v>
       </c>
       <c r="AR292" t="n">
         <v>510.05</v>
@@ -46772,7 +46666,7 @@
         <v>52.5</v>
       </c>
       <c r="AQ293" t="n">
-        <v>52.47</v>
+        <v>52.4</v>
       </c>
       <c r="AR293" t="n">
         <v>1577.68</v>
@@ -46930,7 +46824,7 @@
         <v>51.34</v>
       </c>
       <c r="AQ294" t="n">
-        <v>53.77</v>
+        <v>54.08</v>
       </c>
       <c r="AR294" t="n">
         <v>548.58</v>
@@ -47088,7 +46982,7 @@
         <v>64.02</v>
       </c>
       <c r="AQ295" t="n">
-        <v>58.73</v>
+        <v>58.69</v>
       </c>
       <c r="AR295" t="n">
         <v>418.99</v>
@@ -47246,7 +47140,7 @@
         <v>45.1</v>
       </c>
       <c r="AQ296" t="n">
-        <v>50.62</v>
+        <v>50.61</v>
       </c>
       <c r="AR296" t="n">
         <v>7138.06</v>
@@ -47404,7 +47298,7 @@
         <v>44.38</v>
       </c>
       <c r="AQ297" t="n">
-        <v>65.73999999999999</v>
+        <v>66.22</v>
       </c>
       <c r="AR297" t="n">
         <v>1744.82</v>
@@ -47562,7 +47456,7 @@
         <v>61.4</v>
       </c>
       <c r="AQ298" t="n">
-        <v>52.71</v>
+        <v>52.94</v>
       </c>
       <c r="AR298" t="n">
         <v>923.78</v>
@@ -47720,7 +47614,7 @@
         <v>67.89</v>
       </c>
       <c r="AQ299" t="n">
-        <v>61.32</v>
+        <v>60.71</v>
       </c>
       <c r="AR299" t="n">
         <v>4163.15</v>
@@ -47878,7 +47772,7 @@
         <v>66.09</v>
       </c>
       <c r="AQ300" t="n">
-        <v>57.61</v>
+        <v>57.52</v>
       </c>
       <c r="AR300" t="n">
         <v>289.25</v>
@@ -48036,7 +47930,7 @@
         <v>49.05</v>
       </c>
       <c r="AQ301" t="n">
-        <v>43.67</v>
+        <v>43.35</v>
       </c>
       <c r="AR301" t="n">
         <v>383.76</v>
@@ -48194,7 +48088,7 @@
         <v>36.16</v>
       </c>
       <c r="AQ302" t="n">
-        <v>28.53</v>
+        <v>28.52</v>
       </c>
       <c r="AR302" t="n">
         <v>3851.37</v>
@@ -48352,7 +48246,7 @@
         <v>44.36</v>
       </c>
       <c r="AQ303" t="n">
-        <v>43.25</v>
+        <v>43.46</v>
       </c>
       <c r="AR303" t="n">
         <v>3347.73</v>
@@ -48510,7 +48404,7 @@
         <v>60.06</v>
       </c>
       <c r="AQ304" t="n">
-        <v>61.62</v>
+        <v>62.56</v>
       </c>
       <c r="AR304" t="n">
         <v>2329.51</v>
@@ -48668,7 +48562,7 @@
         <v>62.46</v>
       </c>
       <c r="AQ305" t="n">
-        <v>49.19</v>
+        <v>49.35</v>
       </c>
       <c r="AR305" t="n">
         <v>3092.16</v>
@@ -48826,7 +48720,7 @@
         <v>73.48999999999999</v>
       </c>
       <c r="AQ306" t="n">
-        <v>54.14</v>
+        <v>54.58</v>
       </c>
       <c r="AR306" t="n">
         <v>302.94</v>
@@ -48984,7 +48878,7 @@
         <v>65.3</v>
       </c>
       <c r="AQ307" t="n">
-        <v>72.06999999999999</v>
+        <v>72.25</v>
       </c>
       <c r="AR307" t="n">
         <v>88.04000000000001</v>
@@ -49142,7 +49036,7 @@
         <v>54.12</v>
       </c>
       <c r="AQ308" t="n">
-        <v>60.76</v>
+        <v>60.87</v>
       </c>
       <c r="AR308" t="n">
         <v>317.67</v>
@@ -49300,7 +49194,7 @@
         <v>57.27</v>
       </c>
       <c r="AQ309" t="n">
-        <v>63.84</v>
+        <v>63.82</v>
       </c>
       <c r="AR309" t="n">
         <v>2450.12</v>
@@ -49458,7 +49352,7 @@
         <v>39.44</v>
       </c>
       <c r="AQ310" t="n">
-        <v>31.99</v>
+        <v>31.71</v>
       </c>
       <c r="AR310" t="n">
         <v>866.58</v>
@@ -49616,7 +49510,7 @@
         <v>57.72</v>
       </c>
       <c r="AQ311" t="n">
-        <v>64.04000000000001</v>
+        <v>64.23</v>
       </c>
       <c r="AR311" t="n">
         <v>818.0599999999999</v>
@@ -49774,7 +49668,7 @@
         <v>62.56</v>
       </c>
       <c r="AQ312" t="n">
-        <v>50</v>
+        <v>50.11</v>
       </c>
       <c r="AR312" t="n">
         <v>13460.36</v>
@@ -49932,7 +49826,7 @@
         <v>75.89</v>
       </c>
       <c r="AQ313" t="n">
-        <v>64.31</v>
+        <v>64.27</v>
       </c>
       <c r="AR313" t="n">
         <v>1074.36</v>
@@ -50090,7 +49984,7 @@
         <v>49.2</v>
       </c>
       <c r="AQ314" t="n">
-        <v>49.4</v>
+        <v>48.85</v>
       </c>
       <c r="AR314" t="n">
         <v>2489.17</v>
@@ -50248,7 +50142,7 @@
         <v>42.88</v>
       </c>
       <c r="AQ315" t="n">
-        <v>54.67</v>
+        <v>54.76</v>
       </c>
       <c r="AR315" t="n">
         <v>2842.95</v>
@@ -50406,7 +50300,7 @@
         <v>71.45999999999999</v>
       </c>
       <c r="AQ316" t="n">
-        <v>68.89</v>
+        <v>69.11</v>
       </c>
       <c r="AR316" t="n">
         <v>1281.23</v>
@@ -50564,7 +50458,7 @@
         <v>63.23</v>
       </c>
       <c r="AQ317" t="n">
-        <v>57.06</v>
+        <v>56.78</v>
       </c>
       <c r="AR317" t="n">
         <v>178.55</v>
@@ -50722,7 +50616,7 @@
         <v>45.21</v>
       </c>
       <c r="AQ318" t="n">
-        <v>47.82</v>
+        <v>48.37</v>
       </c>
       <c r="AR318" t="n">
         <v>1646.26</v>
@@ -50880,7 +50774,7 @@
         <v>55.87</v>
       </c>
       <c r="AQ319" t="n">
-        <v>57.01</v>
+        <v>57.56</v>
       </c>
       <c r="AR319" t="n">
         <v>1184.46</v>
@@ -51038,7 +50932,7 @@
         <v>71.09</v>
       </c>
       <c r="AQ320" t="n">
-        <v>72.20999999999999</v>
+        <v>72.26000000000001</v>
       </c>
       <c r="AR320" t="n">
         <v>658.58</v>
@@ -51196,7 +51090,7 @@
         <v>46.5</v>
       </c>
       <c r="AQ321" t="n">
-        <v>55.31</v>
+        <v>55.18</v>
       </c>
       <c r="AR321" t="n">
         <v>71.70999999999999</v>
@@ -51354,7 +51248,7 @@
         <v>67.76000000000001</v>
       </c>
       <c r="AQ322" t="n">
-        <v>72.94</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="AR322" t="n">
         <v>146.04</v>
@@ -51512,7 +51406,7 @@
         <v>64.8</v>
       </c>
       <c r="AQ323" t="n">
-        <v>66.06</v>
+        <v>66.41</v>
       </c>
       <c r="AR323" t="n">
         <v>931.63</v>
@@ -51670,7 +51564,7 @@
         <v>46.18</v>
       </c>
       <c r="AQ324" t="n">
-        <v>45.37</v>
+        <v>45.45</v>
       </c>
       <c r="AR324" t="n">
         <v>2280.05</v>
@@ -51828,7 +51722,7 @@
         <v>57.39</v>
       </c>
       <c r="AQ325" t="n">
-        <v>44.34</v>
+        <v>44.91</v>
       </c>
       <c r="AR325" t="n">
         <v>129208.9</v>
@@ -51986,7 +51880,7 @@
         <v>45.82</v>
       </c>
       <c r="AQ326" t="n">
-        <v>43.36</v>
+        <v>43.01</v>
       </c>
       <c r="AR326" t="n">
         <v>156.35</v>
@@ -52144,7 +52038,7 @@
         <v>69.09</v>
       </c>
       <c r="AQ327" t="n">
-        <v>53.01</v>
+        <v>52.26</v>
       </c>
       <c r="AR327" t="n">
         <v>38.51</v>
@@ -52302,7 +52196,7 @@
         <v>39.39</v>
       </c>
       <c r="AQ328" t="n">
-        <v>36.05</v>
+        <v>35.99</v>
       </c>
       <c r="AR328" t="n">
         <v>3115.14</v>
@@ -52460,7 +52354,7 @@
         <v>57.1</v>
       </c>
       <c r="AQ329" t="n">
-        <v>67.5</v>
+        <v>67.67</v>
       </c>
       <c r="AR329" t="n">
         <v>1139.41</v>
@@ -52618,7 +52512,7 @@
         <v>42.32</v>
       </c>
       <c r="AQ330" t="n">
-        <v>41.13</v>
+        <v>41.28</v>
       </c>
       <c r="AR330" t="n">
         <v>889.92</v>
@@ -52776,7 +52670,7 @@
         <v>25.17</v>
       </c>
       <c r="AQ331" t="n">
-        <v>36.86</v>
+        <v>37.04</v>
       </c>
       <c r="AR331" t="n">
         <v>361.27</v>
@@ -52934,7 +52828,7 @@
         <v>46.18</v>
       </c>
       <c r="AQ332" t="n">
-        <v>38.35</v>
+        <v>38.51</v>
       </c>
       <c r="AR332" t="n">
         <v>994.0599999999999</v>
@@ -53092,7 +52986,7 @@
         <v>48.81</v>
       </c>
       <c r="AQ333" t="n">
-        <v>50.25</v>
+        <v>49.92</v>
       </c>
       <c r="AR333" t="n">
         <v>608.5700000000001</v>
@@ -53250,7 +53144,7 @@
         <v>66.33</v>
       </c>
       <c r="AQ334" t="n">
-        <v>75.84999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="AR334" t="n">
         <v>7468.93</v>
@@ -53408,7 +53302,7 @@
         <v>54.04</v>
       </c>
       <c r="AQ335" t="n">
-        <v>59.02</v>
+        <v>58.8</v>
       </c>
       <c r="AR335" t="n">
         <v>108.35</v>
@@ -53566,7 +53460,7 @@
         <v>51.2</v>
       </c>
       <c r="AQ336" t="n">
-        <v>47.96</v>
+        <v>48.01</v>
       </c>
       <c r="AR336" t="n">
         <v>154.58</v>
@@ -53724,7 +53618,7 @@
         <v>50.18</v>
       </c>
       <c r="AQ337" t="n">
-        <v>59.53</v>
+        <v>61.06</v>
       </c>
       <c r="AR337" t="n">
         <v>1398.04</v>
@@ -53882,7 +53776,7 @@
         <v>58.85</v>
       </c>
       <c r="AQ338" t="n">
-        <v>68.26000000000001</v>
+        <v>68.48</v>
       </c>
       <c r="AR338" t="n">
         <v>4913.09</v>
@@ -54040,7 +53934,7 @@
         <v>66.83</v>
       </c>
       <c r="AQ339" t="n">
-        <v>68.34</v>
+        <v>68.38</v>
       </c>
       <c r="AR339" t="n">
         <v>17562.48</v>
@@ -54198,7 +54092,7 @@
         <v>49.03</v>
       </c>
       <c r="AQ340" t="n">
-        <v>40.47</v>
+        <v>40.53</v>
       </c>
       <c r="AR340" t="n">
         <v>476.15</v>
@@ -54356,7 +54250,7 @@
         <v>61.24</v>
       </c>
       <c r="AQ341" t="n">
-        <v>62.25</v>
+        <v>61.9</v>
       </c>
       <c r="AR341" t="n">
         <v>1916.78</v>
@@ -54514,7 +54408,7 @@
         <v>63.04</v>
       </c>
       <c r="AQ342" t="n">
-        <v>53.69</v>
+        <v>53.31</v>
       </c>
       <c r="AR342" t="n">
         <v>77.25</v>
@@ -54672,7 +54566,7 @@
         <v>58.91</v>
       </c>
       <c r="AQ343" t="n">
-        <v>61.49</v>
+        <v>61.24</v>
       </c>
       <c r="AR343" t="n">
         <v>183.26</v>
@@ -54830,7 +54724,7 @@
         <v>51.87</v>
       </c>
       <c r="AQ344" t="n">
-        <v>61.4</v>
+        <v>62.35</v>
       </c>
       <c r="AR344" t="n">
         <v>85.54000000000001</v>
@@ -54988,7 +54882,7 @@
         <v>44.52</v>
       </c>
       <c r="AQ345" t="n">
-        <v>58.82</v>
+        <v>58.51</v>
       </c>
       <c r="AR345" t="n">
         <v>322.91</v>
@@ -55146,7 +55040,7 @@
         <v>34.9</v>
       </c>
       <c r="AQ346" t="n">
-        <v>49.21</v>
+        <v>48.86</v>
       </c>
       <c r="AR346" t="n">
         <v>87.13</v>
@@ -55304,7 +55198,7 @@
         <v>35.28</v>
       </c>
       <c r="AQ347" t="n">
-        <v>51.45</v>
+        <v>51.51</v>
       </c>
       <c r="AR347" t="n">
         <v>45.81</v>
@@ -55462,7 +55356,7 @@
         <v>34.43</v>
       </c>
       <c r="AQ348" t="n">
-        <v>40.24</v>
+        <v>40.42</v>
       </c>
       <c r="AR348" t="n">
         <v>359.18</v>
@@ -55778,7 +55672,7 @@
         <v>73.78</v>
       </c>
       <c r="AQ350" t="n">
-        <v>70.18000000000001</v>
+        <v>70.61</v>
       </c>
       <c r="AR350" t="n">
         <v>1704.4</v>
@@ -55936,7 +55830,7 @@
         <v>42.77</v>
       </c>
       <c r="AQ351" t="n">
-        <v>43.1</v>
+        <v>43</v>
       </c>
       <c r="AR351" t="n">
         <v>311.73</v>
@@ -56094,7 +55988,7 @@
         <v>70.02</v>
       </c>
       <c r="AQ352" t="n">
-        <v>69.64</v>
+        <v>69.38</v>
       </c>
       <c r="AR352" t="n">
         <v>294.56</v>
@@ -56252,7 +56146,7 @@
         <v>66.78</v>
       </c>
       <c r="AQ353" t="n">
-        <v>61.81</v>
+        <v>62.61</v>
       </c>
       <c r="AR353" t="n">
         <v>1704.68</v>
@@ -56410,7 +56304,7 @@
         <v>77.89</v>
       </c>
       <c r="AQ354" t="n">
-        <v>76.34</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="AR354" t="n">
         <v>10034.44</v>
@@ -56568,7 +56462,7 @@
         <v>24.71</v>
       </c>
       <c r="AQ355" t="n">
-        <v>36.62</v>
+        <v>36.47</v>
       </c>
       <c r="AR355" t="n">
         <v>421.13</v>
@@ -56726,7 +56620,7 @@
         <v>47.11</v>
       </c>
       <c r="AQ356" t="n">
-        <v>58.76</v>
+        <v>58.24</v>
       </c>
       <c r="AR356" t="n">
         <v>42.94</v>
@@ -56884,7 +56778,7 @@
         <v>70.31</v>
       </c>
       <c r="AQ357" t="n">
-        <v>67.7</v>
+        <v>68.95</v>
       </c>
       <c r="AR357" t="n">
         <v>1443.03</v>
@@ -57042,7 +56936,7 @@
         <v>27.79</v>
       </c>
       <c r="AQ358" t="n">
-        <v>43.69</v>
+        <v>42.86</v>
       </c>
       <c r="AR358" t="n">
         <v>1604.32</v>
@@ -57200,7 +57094,7 @@
         <v>17.62</v>
       </c>
       <c r="AQ359" t="n">
-        <v>33.29</v>
+        <v>33.31</v>
       </c>
       <c r="AR359" t="n">
         <v>243.86</v>
@@ -57358,7 +57252,7 @@
         <v>68.39</v>
       </c>
       <c r="AQ360" t="n">
-        <v>68.78</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="AR360" t="n">
         <v>39927.61</v>
@@ -57516,7 +57410,7 @@
         <v>63.07</v>
       </c>
       <c r="AQ361" t="n">
-        <v>57.49</v>
+        <v>57.44</v>
       </c>
       <c r="AR361" t="n">
         <v>134.18</v>
@@ -57674,7 +57568,7 @@
         <v>28.34</v>
       </c>
       <c r="AQ362" t="n">
-        <v>19.04</v>
+        <v>18.56</v>
       </c>
       <c r="AR362" t="n">
         <v>418.64</v>
@@ -57832,7 +57726,7 @@
         <v>58.08</v>
       </c>
       <c r="AQ363" t="n">
-        <v>49.78</v>
+        <v>49.53</v>
       </c>
       <c r="AR363" t="n">
         <v>1096.57</v>
@@ -57990,7 +57884,7 @@
         <v>67.91</v>
       </c>
       <c r="AQ364" t="n">
-        <v>61.62</v>
+        <v>61.44</v>
       </c>
       <c r="AR364" t="n">
         <v>308.48</v>
@@ -58148,7 +58042,7 @@
         <v>42.82</v>
       </c>
       <c r="AQ365" t="n">
-        <v>42.24</v>
+        <v>42.39</v>
       </c>
       <c r="AR365" t="n">
         <v>4901.35</v>
@@ -58306,7 +58200,7 @@
         <v>54.76</v>
       </c>
       <c r="AQ366" t="n">
-        <v>54.83</v>
+        <v>54.69</v>
       </c>
       <c r="AR366" t="n">
         <v>283.81</v>
@@ -58464,7 +58358,7 @@
         <v>51.13</v>
       </c>
       <c r="AQ367" t="n">
-        <v>54.73</v>
+        <v>55.01</v>
       </c>
       <c r="AR367" t="n">
         <v>432.08</v>
@@ -58622,7 +58516,7 @@
         <v>40.13</v>
       </c>
       <c r="AQ368" t="n">
-        <v>38.1</v>
+        <v>38.08</v>
       </c>
       <c r="AR368" t="n">
         <v>4500.23</v>
@@ -58780,7 +58674,7 @@
         <v>61.44</v>
       </c>
       <c r="AQ369" t="n">
-        <v>53.71</v>
+        <v>53.79</v>
       </c>
       <c r="AR369" t="n">
         <v>541.76</v>
@@ -58938,7 +58832,7 @@
         <v>67.31</v>
       </c>
       <c r="AQ370" t="n">
-        <v>65.20999999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="AR370" t="n">
         <v>1864.14</v>
@@ -59096,7 +58990,7 @@
         <v>76.75</v>
       </c>
       <c r="AQ371" t="n">
-        <v>72.53</v>
+        <v>72.42</v>
       </c>
       <c r="AR371" t="n">
         <v>1568.32</v>
@@ -59254,7 +59148,7 @@
         <v>34.25</v>
       </c>
       <c r="AQ372" t="n">
-        <v>33.35</v>
+        <v>33.17</v>
       </c>
       <c r="AR372" t="n">
         <v>2773.88</v>
@@ -59412,7 +59306,7 @@
         <v>59.84</v>
       </c>
       <c r="AQ373" t="n">
-        <v>40.78</v>
+        <v>41.05</v>
       </c>
       <c r="AR373" t="n">
         <v>154.19</v>
@@ -59570,7 +59464,7 @@
         <v>66.31999999999999</v>
       </c>
       <c r="AQ374" t="n">
-        <v>68.64</v>
+        <v>67.67</v>
       </c>
       <c r="AR374" t="n">
         <v>2079.78</v>
@@ -59728,7 +59622,7 @@
         <v>56.92</v>
       </c>
       <c r="AQ375" t="n">
-        <v>49</v>
+        <v>49.06</v>
       </c>
       <c r="AR375" t="n">
         <v>107.73</v>
@@ -59886,7 +59780,7 @@
         <v>61.38</v>
       </c>
       <c r="AQ376" t="n">
-        <v>63.44</v>
+        <v>63.36</v>
       </c>
       <c r="AR376" t="n">
         <v>1020.91</v>
@@ -60044,7 +59938,7 @@
         <v>49.08</v>
       </c>
       <c r="AQ377" t="n">
-        <v>49.43</v>
+        <v>49.17</v>
       </c>
       <c r="AR377" t="n">
         <v>1617.67</v>
@@ -60202,7 +60096,7 @@
         <v>47.56</v>
       </c>
       <c r="AQ378" t="n">
-        <v>64.09999999999999</v>
+        <v>64.53</v>
       </c>
       <c r="AR378" t="n">
         <v>9738.02</v>
@@ -60360,7 +60254,7 @@
         <v>67.55</v>
       </c>
       <c r="AQ379" t="n">
-        <v>57.62</v>
+        <v>57.61</v>
       </c>
       <c r="AR379" t="n">
         <v>1596.43</v>
@@ -60518,7 +60412,7 @@
         <v>74.12</v>
       </c>
       <c r="AQ380" t="n">
-        <v>55.88</v>
+        <v>55.69</v>
       </c>
       <c r="AR380" t="n">
         <v>419.5</v>
@@ -60676,7 +60570,7 @@
         <v>38.81</v>
       </c>
       <c r="AQ381" t="n">
-        <v>42.99</v>
+        <v>43.38</v>
       </c>
       <c r="AR381" t="n">
         <v>288.35</v>
@@ -60834,7 +60728,7 @@
         <v>42.04</v>
       </c>
       <c r="AQ382" t="n">
-        <v>59.65</v>
+        <v>59.73</v>
       </c>
       <c r="AR382" t="n">
         <v>35175.02</v>
@@ -60992,7 +60886,7 @@
         <v>51.98</v>
       </c>
       <c r="AQ383" t="n">
-        <v>52.64</v>
+        <v>52.45</v>
       </c>
       <c r="AR383" t="n">
         <v>165.84</v>
@@ -61150,7 +61044,7 @@
         <v>49.5</v>
       </c>
       <c r="AQ384" t="n">
-        <v>60.77</v>
+        <v>59.91</v>
       </c>
       <c r="AR384" t="n">
         <v>1056.16</v>
@@ -61308,7 +61202,7 @@
         <v>71.15000000000001</v>
       </c>
       <c r="AQ385" t="n">
-        <v>61.37</v>
+        <v>61.48</v>
       </c>
       <c r="AR385" t="n">
         <v>1504.29</v>
@@ -61466,7 +61360,7 @@
         <v>45.57</v>
       </c>
       <c r="AQ386" t="n">
-        <v>52.29</v>
+        <v>52.33</v>
       </c>
       <c r="AR386" t="n">
         <v>17759.58</v>
@@ -61624,7 +61518,7 @@
         <v>58.3</v>
       </c>
       <c r="AQ387" t="n">
-        <v>48.11</v>
+        <v>47.34</v>
       </c>
       <c r="AR387" t="n">
         <v>971.72</v>
@@ -61782,7 +61676,7 @@
         <v>67.7</v>
       </c>
       <c r="AQ388" t="n">
-        <v>65.93000000000001</v>
+        <v>64.64</v>
       </c>
       <c r="AR388" t="n">
         <v>120.57</v>
@@ -61940,7 +61834,7 @@
         <v>73.84</v>
       </c>
       <c r="AQ389" t="n">
-        <v>79.17</v>
+        <v>79.12</v>
       </c>
       <c r="AR389" t="n">
         <v>3707.67</v>
@@ -62098,7 +61992,7 @@
         <v>46.86</v>
       </c>
       <c r="AQ390" t="n">
-        <v>48.8</v>
+        <v>48.41</v>
       </c>
       <c r="AR390" t="n">
         <v>317.35</v>
@@ -62256,7 +62150,7 @@
         <v>64.34999999999999</v>
       </c>
       <c r="AQ391" t="n">
-        <v>67.28</v>
+        <v>66.69</v>
       </c>
       <c r="AR391" t="n">
         <v>1428.38</v>
@@ -62414,7 +62308,7 @@
         <v>60.94</v>
       </c>
       <c r="AQ392" t="n">
-        <v>43.3</v>
+        <v>42.88</v>
       </c>
       <c r="AR392" t="n">
         <v>894.58</v>
@@ -62572,7 +62466,7 @@
         <v>59.02</v>
       </c>
       <c r="AQ393" t="n">
-        <v>68.93000000000001</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="AR393" t="n">
         <v>371.06</v>
@@ -62730,7 +62624,7 @@
         <v>61.92</v>
       </c>
       <c r="AQ394" t="n">
-        <v>58.74</v>
+        <v>58.63</v>
       </c>
       <c r="AR394" t="n">
         <v>359.45</v>
@@ -62888,7 +62782,7 @@
         <v>77.59</v>
       </c>
       <c r="AQ395" t="n">
-        <v>68.83</v>
+        <v>68.48</v>
       </c>
       <c r="AR395" t="n">
         <v>270.33</v>
@@ -63046,7 +62940,7 @@
         <v>51.21</v>
       </c>
       <c r="AQ396" t="n">
-        <v>42.38</v>
+        <v>42.09</v>
       </c>
       <c r="AR396" t="n">
         <v>1313.64</v>
@@ -63204,7 +63098,7 @@
         <v>46.96</v>
       </c>
       <c r="AQ397" t="n">
-        <v>41.25</v>
+        <v>40.92</v>
       </c>
       <c r="AR397" t="n">
         <v>379.06</v>
@@ -63362,7 +63256,7 @@
         <v>50.94</v>
       </c>
       <c r="AQ398" t="n">
-        <v>47.3</v>
+        <v>46.97</v>
       </c>
       <c r="AR398" t="n">
         <v>209.43</v>
@@ -63520,7 +63414,7 @@
         <v>43.64</v>
       </c>
       <c r="AQ399" t="n">
-        <v>51.63</v>
+        <v>51.49</v>
       </c>
       <c r="AR399" t="n">
         <v>575.35</v>
@@ -63836,7 +63730,7 @@
         <v>85.41</v>
       </c>
       <c r="AQ401" t="n">
-        <v>83.95</v>
+        <v>83.98</v>
       </c>
       <c r="AR401" t="n">
         <v>2340.06</v>
@@ -63994,7 +63888,7 @@
         <v>44.35</v>
       </c>
       <c r="AQ402" t="n">
-        <v>33.56</v>
+        <v>33.51</v>
       </c>
       <c r="AR402" t="n">
         <v>241.22</v>
@@ -64152,7 +64046,7 @@
         <v>50.86</v>
       </c>
       <c r="AQ403" t="n">
-        <v>40.19</v>
+        <v>40.33</v>
       </c>
       <c r="AR403" t="n">
         <v>40.03</v>
@@ -64310,7 +64204,7 @@
         <v>30.15</v>
       </c>
       <c r="AQ404" t="n">
-        <v>48.03</v>
+        <v>47.69</v>
       </c>
       <c r="AR404" t="n">
         <v>176.27</v>
@@ -64468,7 +64362,7 @@
         <v>60.66</v>
       </c>
       <c r="AQ405" t="n">
-        <v>75.25</v>
+        <v>75</v>
       </c>
       <c r="AR405" t="n">
         <v>1208.56</v>
@@ -64626,7 +64520,7 @@
         <v>46.36</v>
       </c>
       <c r="AQ406" t="n">
-        <v>57.5</v>
+        <v>57.25</v>
       </c>
       <c r="AR406" t="n">
         <v>173.82</v>
@@ -64784,7 +64678,7 @@
         <v>48.64</v>
       </c>
       <c r="AQ407" t="n">
-        <v>45.7</v>
+        <v>44.9</v>
       </c>
       <c r="AR407" t="n">
         <v>183.31</v>
@@ -64942,7 +64836,7 @@
         <v>44.2</v>
       </c>
       <c r="AQ408" t="n">
-        <v>46.23</v>
+        <v>46.21</v>
       </c>
       <c r="AR408" t="n">
         <v>522.3</v>
@@ -65100,7 +64994,7 @@
         <v>66.98</v>
       </c>
       <c r="AQ409" t="n">
-        <v>73.56</v>
+        <v>73.5</v>
       </c>
       <c r="AR409" t="n">
         <v>468.04</v>
@@ -65258,7 +65152,7 @@
         <v>45.91</v>
       </c>
       <c r="AQ410" t="n">
-        <v>45.24</v>
+        <v>45.28</v>
       </c>
       <c r="AR410" t="n">
         <v>91.89</v>
@@ -65416,7 +65310,7 @@
         <v>56.68</v>
       </c>
       <c r="AQ411" t="n">
-        <v>35.92</v>
+        <v>35.84</v>
       </c>
       <c r="AR411" t="n">
         <v>613.75</v>
@@ -65574,7 +65468,7 @@
         <v>38.29</v>
       </c>
       <c r="AQ412" t="n">
-        <v>39.73</v>
+        <v>39.54</v>
       </c>
       <c r="AR412" t="n">
         <v>1774.23</v>
@@ -65732,7 +65626,7 @@
         <v>66.95</v>
       </c>
       <c r="AQ413" t="n">
-        <v>55.63</v>
+        <v>55.6</v>
       </c>
       <c r="AR413" t="n">
         <v>1029.29</v>
@@ -65890,7 +65784,7 @@
         <v>50.89</v>
       </c>
       <c r="AQ414" t="n">
-        <v>53.55</v>
+        <v>53.33</v>
       </c>
       <c r="AR414" t="n">
         <v>4193.11</v>
@@ -66048,7 +65942,7 @@
         <v>57.18</v>
       </c>
       <c r="AQ415" t="n">
-        <v>67.37</v>
+        <v>67.97</v>
       </c>
       <c r="AR415" t="n">
         <v>1318.26</v>
@@ -66206,7 +66100,7 @@
         <v>52.06</v>
       </c>
       <c r="AQ416" t="n">
-        <v>60.41</v>
+        <v>60.7</v>
       </c>
       <c r="AR416" t="n">
         <v>313.39</v>
@@ -66364,7 +66258,7 @@
         <v>62.64</v>
       </c>
       <c r="AQ417" t="n">
-        <v>54.52</v>
+        <v>54.71</v>
       </c>
       <c r="AR417" t="n">
         <v>25223.65</v>
@@ -66522,7 +66416,7 @@
         <v>70.3</v>
       </c>
       <c r="AQ418" t="n">
-        <v>59.47</v>
+        <v>59.37</v>
       </c>
       <c r="AR418" t="n">
         <v>997.87</v>
@@ -66680,7 +66574,7 @@
         <v>43.37</v>
       </c>
       <c r="AQ419" t="n">
-        <v>58.5</v>
+        <v>58.37</v>
       </c>
       <c r="AR419" t="n">
         <v>960.24</v>
@@ -66838,7 +66732,7 @@
         <v>46.19</v>
       </c>
       <c r="AQ420" t="n">
-        <v>54.31</v>
+        <v>54.51</v>
       </c>
       <c r="AR420" t="n">
         <v>3661.75</v>
@@ -66996,7 +66890,7 @@
         <v>30.02</v>
       </c>
       <c r="AQ421" t="n">
-        <v>36.94</v>
+        <v>37.35</v>
       </c>
       <c r="AR421" t="n">
         <v>782.63</v>
@@ -67154,7 +67048,7 @@
         <v>42.88</v>
       </c>
       <c r="AQ422" t="n">
-        <v>43.62</v>
+        <v>43.82</v>
       </c>
       <c r="AR422" t="n">
         <v>73</v>
@@ -67312,7 +67206,7 @@
         <v>55.69</v>
       </c>
       <c r="AQ423" t="n">
-        <v>51.48</v>
+        <v>50.95</v>
       </c>
       <c r="AR423" t="n">
         <v>1401.17</v>
@@ -67470,7 +67364,7 @@
         <v>45.2</v>
       </c>
       <c r="AQ424" t="n">
-        <v>62.19</v>
+        <v>62.21</v>
       </c>
       <c r="AR424" t="n">
         <v>17800.28</v>
@@ -67628,7 +67522,7 @@
         <v>63.68</v>
       </c>
       <c r="AQ425" t="n">
-        <v>66.47</v>
+        <v>66.48999999999999</v>
       </c>
       <c r="AR425" t="n">
         <v>610.6900000000001</v>
@@ -67786,7 +67680,7 @@
         <v>52.51</v>
       </c>
       <c r="AQ426" t="n">
-        <v>51.87</v>
+        <v>51.8</v>
       </c>
       <c r="AR426" t="n">
         <v>287.99</v>
@@ -67944,7 +67838,7 @@
         <v>58.56</v>
       </c>
       <c r="AQ427" t="n">
-        <v>55.96</v>
+        <v>56.71</v>
       </c>
       <c r="AR427" t="n">
         <v>735.9</v>
@@ -68102,7 +67996,7 @@
         <v>53.54</v>
       </c>
       <c r="AQ428" t="n">
-        <v>54.01</v>
+        <v>53.94</v>
       </c>
       <c r="AR428" t="n">
         <v>2728.74</v>
@@ -68260,7 +68154,7 @@
         <v>72.67</v>
       </c>
       <c r="AQ429" t="n">
-        <v>73.28</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="AR429" t="n">
         <v>563.97</v>
@@ -68418,7 +68312,7 @@
         <v>37.58</v>
       </c>
       <c r="AQ430" t="n">
-        <v>47.15</v>
+        <v>47.09</v>
       </c>
       <c r="AR430" t="n">
         <v>448.12</v>
@@ -68576,7 +68470,7 @@
         <v>65.97</v>
       </c>
       <c r="AQ431" t="n">
-        <v>49.68</v>
+        <v>49.61</v>
       </c>
       <c r="AR431" t="n">
         <v>4489.33</v>
@@ -68734,7 +68628,7 @@
         <v>65.34999999999999</v>
       </c>
       <c r="AQ432" t="n">
-        <v>61.15</v>
+        <v>61.03</v>
       </c>
       <c r="AR432" t="n">
         <v>1845.28</v>
@@ -68892,7 +68786,7 @@
         <v>44.36</v>
       </c>
       <c r="AQ433" t="n">
-        <v>40.78</v>
+        <v>40.71</v>
       </c>
       <c r="AR433" t="n">
         <v>517.26</v>
@@ -69050,7 +68944,7 @@
         <v>39.52</v>
       </c>
       <c r="AQ434" t="n">
-        <v>38.27</v>
+        <v>38.36</v>
       </c>
       <c r="AR434" t="n">
         <v>3499.13</v>
@@ -69208,7 +69102,7 @@
         <v>53.24</v>
       </c>
       <c r="AQ435" t="n">
-        <v>62.07</v>
+        <v>61.68</v>
       </c>
       <c r="AR435" t="n">
         <v>57.64</v>
@@ -69366,7 +69260,7 @@
         <v>47.79</v>
       </c>
       <c r="AQ436" t="n">
-        <v>37.27</v>
+        <v>36.96</v>
       </c>
       <c r="AR436" t="n">
         <v>320.93</v>
@@ -69524,7 +69418,7 @@
         <v>36.81</v>
       </c>
       <c r="AQ437" t="n">
-        <v>28.04</v>
+        <v>27.93</v>
       </c>
       <c r="AR437" t="n">
         <v>249.31</v>
@@ -69682,7 +69576,7 @@
         <v>42.89</v>
       </c>
       <c r="AQ438" t="n">
-        <v>42.13</v>
+        <v>42.34</v>
       </c>
       <c r="AR438" t="n">
         <v>441.42</v>
@@ -69840,7 +69734,7 @@
         <v>85.42</v>
       </c>
       <c r="AQ439" t="n">
-        <v>82.81999999999999</v>
+        <v>82.70999999999999</v>
       </c>
       <c r="AR439" t="n">
         <v>1354.97</v>
@@ -69998,7 +69892,7 @@
         <v>55.02</v>
       </c>
       <c r="AQ440" t="n">
-        <v>55.47</v>
+        <v>55.04</v>
       </c>
       <c r="AR440" t="n">
         <v>335.35</v>
@@ -70156,7 +70050,7 @@
         <v>71.86</v>
       </c>
       <c r="AQ441" t="n">
-        <v>65.64</v>
+        <v>65.22</v>
       </c>
       <c r="AR441" t="n">
         <v>349.58</v>
@@ -70314,7 +70208,7 @@
         <v>58.97</v>
       </c>
       <c r="AQ442" t="n">
-        <v>53.93</v>
+        <v>53.72</v>
       </c>
       <c r="AR442" t="n">
         <v>733.49</v>
@@ -70472,7 +70366,7 @@
         <v>58.54</v>
       </c>
       <c r="AQ443" t="n">
-        <v>75.84</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="AR443" t="n">
         <v>1984.53</v>
@@ -70630,7 +70524,7 @@
         <v>51.95</v>
       </c>
       <c r="AQ444" t="n">
-        <v>49.9</v>
+        <v>49.93</v>
       </c>
       <c r="AR444" t="n">
         <v>1115.17</v>
@@ -70788,7 +70682,7 @@
         <v>40.12</v>
       </c>
       <c r="AQ445" t="n">
-        <v>37.51</v>
+        <v>37.55</v>
       </c>
       <c r="AR445" t="n">
         <v>4075.33</v>
@@ -70946,7 +70840,7 @@
         <v>52.59</v>
       </c>
       <c r="AQ446" t="n">
-        <v>50.9</v>
+        <v>50.26</v>
       </c>
       <c r="AR446" t="n">
         <v>677.23</v>
@@ -71104,7 +70998,7 @@
         <v>33.52</v>
       </c>
       <c r="AQ447" t="n">
-        <v>45.02</v>
+        <v>44.87</v>
       </c>
       <c r="AR447" t="n">
         <v>396.7</v>
@@ -71262,7 +71156,7 @@
         <v>28.33</v>
       </c>
       <c r="AQ448" t="n">
-        <v>42.6</v>
+        <v>42.53</v>
       </c>
       <c r="AR448" t="n">
         <v>194.84</v>
@@ -71420,7 +71314,7 @@
         <v>57.54</v>
       </c>
       <c r="AQ449" t="n">
-        <v>72.09999999999999</v>
+        <v>71.59</v>
       </c>
       <c r="AR449" t="n">
         <v>749.54</v>
@@ -71578,7 +71472,7 @@
         <v>69.37</v>
       </c>
       <c r="AQ450" t="n">
-        <v>62.47</v>
+        <v>62.19</v>
       </c>
       <c r="AR450" t="n">
         <v>1428.8</v>
@@ -71736,7 +71630,7 @@
         <v>37.46</v>
       </c>
       <c r="AQ451" t="n">
-        <v>23.87</v>
+        <v>23.92</v>
       </c>
       <c r="AR451" t="n">
         <v>2131.73</v>
@@ -71894,7 +71788,7 @@
         <v>47.35</v>
       </c>
       <c r="AQ452" t="n">
-        <v>48.56</v>
+        <v>48.83</v>
       </c>
       <c r="AR452" t="n">
         <v>1442.46</v>
@@ -72052,7 +71946,7 @@
         <v>50.23</v>
       </c>
       <c r="AQ453" t="n">
-        <v>46.31</v>
+        <v>46.53</v>
       </c>
       <c r="AR453" t="n">
         <v>1076.89</v>
@@ -72210,7 +72104,7 @@
         <v>46.25</v>
       </c>
       <c r="AQ454" t="n">
-        <v>48.56</v>
+        <v>48.54</v>
       </c>
       <c r="AR454" t="n">
         <v>1760.72</v>
@@ -72368,7 +72262,7 @@
         <v>68.05</v>
       </c>
       <c r="AQ455" t="n">
-        <v>70.14</v>
+        <v>69.58</v>
       </c>
       <c r="AR455" t="n">
         <v>609.75</v>
@@ -72684,7 +72578,7 @@
         <v>70.75</v>
       </c>
       <c r="AQ457" t="n">
-        <v>68.98999999999999</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="AR457" t="n">
         <v>472.51</v>
@@ -72842,7 +72736,7 @@
         <v>57.55</v>
       </c>
       <c r="AQ458" t="n">
-        <v>73.2</v>
+        <v>73.45</v>
       </c>
       <c r="AR458" t="n">
         <v>4772.42</v>
@@ -73000,7 +72894,7 @@
         <v>41.91</v>
       </c>
       <c r="AQ459" t="n">
-        <v>56.73</v>
+        <v>57.02</v>
       </c>
       <c r="AR459" t="n">
         <v>3185.96</v>
@@ -73158,7 +73052,7 @@
         <v>52.56</v>
       </c>
       <c r="AQ460" t="n">
-        <v>59.28</v>
+        <v>59.46</v>
       </c>
       <c r="AR460" t="n">
         <v>3672.71</v>
@@ -73316,7 +73210,7 @@
         <v>54.97</v>
       </c>
       <c r="AQ461" t="n">
-        <v>63.03</v>
+        <v>63.44</v>
       </c>
       <c r="AR461" t="n">
         <v>899.52</v>
@@ -73474,7 +73368,7 @@
         <v>53.25</v>
       </c>
       <c r="AQ462" t="n">
-        <v>53.07</v>
+        <v>53.02</v>
       </c>
       <c r="AR462" t="n">
         <v>4307.16</v>
@@ -73632,7 +73526,7 @@
         <v>72.06</v>
       </c>
       <c r="AQ463" t="n">
-        <v>57.24</v>
+        <v>57.26</v>
       </c>
       <c r="AR463" t="n">
         <v>406.19</v>
@@ -73790,7 +73684,7 @@
         <v>38.42</v>
       </c>
       <c r="AQ464" t="n">
-        <v>47.6</v>
+        <v>47.39</v>
       </c>
       <c r="AR464" t="n">
         <v>361.93</v>
@@ -73948,7 +73842,7 @@
         <v>57.88</v>
       </c>
       <c r="AQ465" t="n">
-        <v>63.84</v>
+        <v>63.98</v>
       </c>
       <c r="AR465" t="n">
         <v>4484.78</v>
@@ -74264,7 +74158,7 @@
         <v>61.59</v>
       </c>
       <c r="AQ467" t="n">
-        <v>59.09</v>
+        <v>59.62</v>
       </c>
       <c r="AR467" t="n">
         <v>1320.39</v>
@@ -74422,7 +74316,7 @@
         <v>71.51000000000001</v>
       </c>
       <c r="AQ468" t="n">
-        <v>61.53</v>
+        <v>61.48</v>
       </c>
       <c r="AR468" t="n">
         <v>3113.91</v>
@@ -74580,7 +74474,7 @@
         <v>66.59999999999999</v>
       </c>
       <c r="AQ469" t="n">
-        <v>59.87</v>
+        <v>59.6</v>
       </c>
       <c r="AR469" t="n">
         <v>25.77</v>
@@ -74738,7 +74632,7 @@
         <v>48.68</v>
       </c>
       <c r="AQ470" t="n">
-        <v>67.04000000000001</v>
+        <v>66.12</v>
       </c>
       <c r="AR470" t="n">
         <v>683.9299999999999</v>
@@ -74896,7 +74790,7 @@
         <v>43.76</v>
       </c>
       <c r="AQ471" t="n">
-        <v>47.08</v>
+        <v>46.85</v>
       </c>
       <c r="AR471" t="n">
         <v>43.81</v>
@@ -75054,7 +74948,7 @@
         <v>65.29000000000001</v>
       </c>
       <c r="AQ472" t="n">
-        <v>52.27</v>
+        <v>52.58</v>
       </c>
       <c r="AR472" t="n">
         <v>3461.53</v>
@@ -75212,7 +75106,7 @@
         <v>43.24</v>
       </c>
       <c r="AQ473" t="n">
-        <v>31.41</v>
+        <v>31.52</v>
       </c>
       <c r="AR473" t="n">
         <v>1336.76</v>
@@ -75370,7 +75264,7 @@
         <v>58.93</v>
       </c>
       <c r="AQ474" t="n">
-        <v>54.21</v>
+        <v>54.35</v>
       </c>
       <c r="AR474" t="n">
         <v>27</v>
@@ -75528,7 +75422,7 @@
         <v>57.81</v>
       </c>
       <c r="AQ475" t="n">
-        <v>48.74</v>
+        <v>48.2</v>
       </c>
       <c r="AR475" t="n">
         <v>11360.62</v>
@@ -75686,7 +75580,7 @@
         <v>60.25</v>
       </c>
       <c r="AQ476" t="n">
-        <v>53.66</v>
+        <v>53.5</v>
       </c>
       <c r="AR476" t="n">
         <v>173.77</v>
@@ -75844,7 +75738,7 @@
         <v>71.94</v>
       </c>
       <c r="AQ477" t="n">
-        <v>58.61</v>
+        <v>58.71</v>
       </c>
       <c r="AR477" t="n">
         <v>1334.98</v>
@@ -76002,7 +75896,7 @@
         <v>59.81</v>
       </c>
       <c r="AQ478" t="n">
-        <v>52.15</v>
+        <v>52.22</v>
       </c>
       <c r="AR478" t="n">
         <v>1109.77</v>
@@ -76160,7 +76054,7 @@
         <v>30.08</v>
       </c>
       <c r="AQ479" t="n">
-        <v>35.19</v>
+        <v>34.94</v>
       </c>
       <c r="AR479" t="n">
         <v>604.38</v>
@@ -76318,7 +76212,7 @@
         <v>52.66</v>
       </c>
       <c r="AQ480" t="n">
-        <v>51.7</v>
+        <v>51.86</v>
       </c>
       <c r="AR480" t="n">
         <v>130.72</v>
@@ -76476,7 +76370,7 @@
         <v>43.47</v>
       </c>
       <c r="AQ481" t="n">
-        <v>56.05</v>
+        <v>56.89</v>
       </c>
       <c r="AR481" t="n">
         <v>479.14</v>
@@ -76634,7 +76528,7 @@
         <v>48.8</v>
       </c>
       <c r="AQ482" t="n">
-        <v>40.77</v>
+        <v>40.59</v>
       </c>
       <c r="AR482" t="n">
         <v>939.72</v>
@@ -76792,7 +76686,7 @@
         <v>39.01</v>
       </c>
       <c r="AQ483" t="n">
-        <v>56.41</v>
+        <v>56.21</v>
       </c>
       <c r="AR483" t="n">
         <v>517.73</v>
@@ -77108,7 +77002,7 @@
         <v>61.57</v>
       </c>
       <c r="AQ485" t="n">
-        <v>68.55</v>
+        <v>68.61</v>
       </c>
       <c r="AR485" t="n">
         <v>1321.51</v>
@@ -77266,7 +77160,7 @@
         <v>40.47</v>
       </c>
       <c r="AQ486" t="n">
-        <v>42.48</v>
+        <v>42.72</v>
       </c>
       <c r="AR486" t="n">
         <v>118.2</v>
@@ -77424,7 +77318,7 @@
         <v>47.7</v>
       </c>
       <c r="AQ487" t="n">
-        <v>46.52</v>
+        <v>46.59</v>
       </c>
       <c r="AR487" t="n">
         <v>1320.16</v>
@@ -77582,7 +77476,7 @@
         <v>52.27</v>
       </c>
       <c r="AQ488" t="n">
-        <v>65.23</v>
+        <v>65.14</v>
       </c>
       <c r="AR488" t="n">
         <v>639.92</v>
@@ -77740,7 +77634,7 @@
         <v>40.42</v>
       </c>
       <c r="AQ489" t="n">
-        <v>47.34</v>
+        <v>47.37</v>
       </c>
       <c r="AR489" t="n">
         <v>3045.81</v>
@@ -77898,7 +77792,7 @@
         <v>65.77</v>
       </c>
       <c r="AQ490" t="n">
-        <v>87.73</v>
+        <v>87.84</v>
       </c>
       <c r="AR490" t="n">
         <v>1412.08</v>
@@ -78056,7 +77950,7 @@
         <v>75.3</v>
       </c>
       <c r="AQ491" t="n">
-        <v>75.93000000000001</v>
+        <v>75.81</v>
       </c>
       <c r="AR491" t="n">
         <v>159.36</v>
@@ -78214,7 +78108,7 @@
         <v>46.56</v>
       </c>
       <c r="AQ492" t="n">
-        <v>38.1</v>
+        <v>38.51</v>
       </c>
       <c r="AR492" t="n">
         <v>801.03</v>
@@ -78372,7 +78266,7 @@
         <v>28.96</v>
       </c>
       <c r="AQ493" t="n">
-        <v>28.29</v>
+        <v>28.33</v>
       </c>
       <c r="AR493" t="n">
         <v>179.05</v>
@@ -78530,7 +78424,7 @@
         <v>55.94</v>
       </c>
       <c r="AQ494" t="n">
-        <v>72.43000000000001</v>
+        <v>72.42</v>
       </c>
       <c r="AR494" t="n">
         <v>1973.66</v>
@@ -78688,7 +78582,7 @@
         <v>63.48</v>
       </c>
       <c r="AQ495" t="n">
-        <v>67.72</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="AR495" t="n">
         <v>24.59</v>
@@ -78846,7 +78740,7 @@
         <v>58.19</v>
       </c>
       <c r="AQ496" t="n">
-        <v>66.98999999999999</v>
+        <v>66.34999999999999</v>
       </c>
       <c r="AR496" t="n">
         <v>112.17</v>
@@ -79004,7 +78898,7 @@
         <v>37.11</v>
       </c>
       <c r="AQ497" t="n">
-        <v>24.44</v>
+        <v>24.39</v>
       </c>
       <c r="AR497" t="n">
         <v>453.14</v>
@@ -79162,7 +79056,7 @@
         <v>46.51</v>
       </c>
       <c r="AQ498" t="n">
-        <v>59.93</v>
+        <v>60.11</v>
       </c>
       <c r="AR498" t="n">
         <v>1857.11</v>
@@ -79320,7 +79214,7 @@
         <v>61.49</v>
       </c>
       <c r="AQ499" t="n">
-        <v>64.17</v>
+        <v>63.51</v>
       </c>
       <c r="AR499" t="n">
         <v>2590.11</v>
@@ -79478,7 +79372,7 @@
         <v>60.57</v>
       </c>
       <c r="AQ500" t="n">
-        <v>70.86</v>
+        <v>70.92</v>
       </c>
       <c r="AR500" t="n">
         <v>1091.93</v>
@@ -79636,7 +79530,7 @@
         <v>54.48</v>
       </c>
       <c r="AQ501" t="n">
-        <v>65.63</v>
+        <v>67.36</v>
       </c>
       <c r="AR501" t="n">
         <v>517.8200000000001</v>

</xml_diff>

<commit_message>
data: nifty500 scan 2026-06-26 09:46 IST
</commit_message>
<xml_diff>
--- a/data/nifty500_latest.xlsx
+++ b/data/nifty500_latest.xlsx
@@ -812,51 +812,157 @@
           <t>3MINDIA.NS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Diversified</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>33225</v>
+      </c>
+      <c r="F3" t="n">
+        <v>33225</v>
+      </c>
+      <c r="G3" t="n">
+        <v>32810</v>
+      </c>
+      <c r="H3" t="n">
+        <v>32560</v>
+      </c>
+      <c r="I3" t="n">
+        <v>32610</v>
+      </c>
+      <c r="J3" t="n">
+        <v>32445</v>
+      </c>
+      <c r="K3" t="n">
+        <v>32290</v>
+      </c>
+      <c r="L3" t="n">
+        <v>31995</v>
+      </c>
+      <c r="M3" t="n">
+        <v>31540</v>
+      </c>
+      <c r="N3" t="n">
+        <v>31785</v>
+      </c>
+      <c r="O3" t="n">
+        <v>31580</v>
+      </c>
+      <c r="P3" t="n">
+        <v>31165</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>31550</v>
+      </c>
+      <c r="R3" t="n">
+        <v>31665</v>
+      </c>
+      <c r="S3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="T3" t="n">
+        <v>33060</v>
+      </c>
+      <c r="U3" t="n">
+        <v>33250</v>
+      </c>
+      <c r="V3" t="n">
+        <v>33125</v>
+      </c>
+      <c r="W3" t="n">
+        <v>33325</v>
+      </c>
+      <c r="X3" t="n">
+        <v>33615</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>33535</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>33380</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>32507.38</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>33615</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>31165</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Between</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Shooting Star</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
       <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
+      <c r="AO3" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>62.21</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>33070.11</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>32265.96</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>2.49</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
data: nifty500 scan 2026-06-26 11:01 IST
</commit_message>
<xml_diff>
--- a/data/nifty500_latest.xlsx
+++ b/data/nifty500_latest.xlsx
@@ -2708,157 +2708,51 @@
           <t>ACC.NS</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Construction Materials</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1418.39</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1418.39</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1391.25</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1352.18</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1362.02</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1343.13</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1343.03</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1322.15</v>
-      </c>
-      <c r="M15" t="n">
-        <v>1312.11</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1317.08</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1308.63</v>
-      </c>
-      <c r="P15" t="n">
-        <v>1296.2</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>1336.6</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1356.4</v>
-      </c>
-      <c r="S15" t="n">
-        <v>1349</v>
-      </c>
-      <c r="T15" t="n">
-        <v>1350</v>
-      </c>
-      <c r="U15" t="n">
-        <v>1358.9</v>
-      </c>
-      <c r="V15" t="n">
-        <v>1343.3</v>
-      </c>
-      <c r="W15" t="n">
-        <v>1349.8</v>
-      </c>
-      <c r="X15" t="n">
-        <v>1329.4</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>1347</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>1337.9</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>1347.85</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>-0.74</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>1418.39</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>1296.2</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>-5.67</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>3.22</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>9.43</v>
-      </c>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>Between</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>Bearish Marubozu</t>
-        </is>
-      </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>Doji</t>
-        </is>
-      </c>
-      <c r="AL15" t="inlineStr">
-        <is>
-          <t>Bearish Marubozu</t>
-        </is>
-      </c>
-      <c r="AM15" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
-      <c r="AO15" t="n">
-        <v>-0.68</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>46.93</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>33.21</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>1341.83</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>1353.27</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>-0.85</v>
-      </c>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">

</xml_diff>

<commit_message>
data: nifty500 scan 2026-06-26 11:16 IST
</commit_message>
<xml_diff>
--- a/data/nifty500_latest.xlsx
+++ b/data/nifty500_latest.xlsx
@@ -2708,51 +2708,157 @@
           <t>ACC.NS</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Construction Materials</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1418.39</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1418.39</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1391.25</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1352.18</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1362.02</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1343.13</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1343.03</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1322.15</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1312.11</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1317.08</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1308.63</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1296.2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1336.6</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1356.4</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1349</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1350</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1358.9</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1343.3</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1349.8</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1329.4</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>1347</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>1337.9</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1347.85</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>1418.39</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>1296.2</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>-5.67</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>Between</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Bearish Marubozu</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>Bearish Marubozu</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
       <c r="AN15" t="inlineStr"/>
-      <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr"/>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr"/>
-      <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
+      <c r="AO15" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>33.21</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>1341.83</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>1353.27</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>-0.85</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">

</xml_diff>